<commit_message>
Avances: Minería de datos
Práctica 5 (Iniciada)
Práctica 6 (Preguntar)
Práctica 7 (Recursos añadidos)
</commit_message>
<xml_diff>
--- a/Minería de datos/Práctica 5/ca_cest_brandi_carlile (Editable).xlsx
+++ b/Minería de datos/Práctica 5/ca_cest_brandi_carlile (Editable).xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repositories\Semestre-EneJun2026\Minería de datos\Práctica 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{7CAD82CC-3098-4D52-A240-559644177B2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3590779-F7A7-4F3E-9859-2D94FC2A9035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6B0EAA5F-3816-4796-860C-BD0B64EC5768}"/>
   </bookViews>
   <sheets>
     <sheet name="ca_cest_brandi_carlile - copia" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
   <si>
     <t>MIN:</t>
   </si>
@@ -62,6 +75,33 @@
   </si>
   <si>
     <t>Tempo</t>
+  </si>
+  <si>
+    <t>Duda:</t>
+  </si>
+  <si>
+    <t>¿Es normal que los datos de Loudness los estemos trabajando como positivos?</t>
+  </si>
+  <si>
+    <t>¿Cuántas veces repito esto?</t>
+  </si>
+  <si>
+    <t>DC0</t>
+  </si>
+  <si>
+    <t>DC1</t>
+  </si>
+  <si>
+    <t>Distancia aeuclidian: Resta de las coordenadas de ambos puntos en la misma dimensión al cuadrado, sumada a tra´ves de todas las dimensiones en raíz</t>
+  </si>
+  <si>
+    <t>dcmin</t>
+  </si>
+  <si>
+    <t>c0</t>
+  </si>
+  <si>
+    <t>c1</t>
   </si>
 </sst>
 </file>
@@ -545,8 +585,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -922,10 +963,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9653E2FD-8EE4-4C35-A4F1-EC87F3E3C160}">
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:AG59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="22" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="14" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="30" max="37" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="14.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -977,8 +1034,63 @@
         <f t="shared" si="0"/>
         <v>69.045000000000002</v>
       </c>
+      <c r="O1" t="s">
+        <v>0</v>
+      </c>
+      <c r="P1">
+        <f>MIN(P5:P55)</f>
+        <v>0</v>
+      </c>
+      <c r="Q1">
+        <f t="shared" ref="Q1:AA1" si="1">MIN(Q5:Q55)</f>
+        <v>0</v>
+      </c>
+      <c r="R1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="S1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="W1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="X1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Z1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AA1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF1">
+        <f>(SUMPRODUCT(P5:P55,AF5:AF55)+P1)/(AF56+1)</f>
+        <v>0.39292103294304903</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -987,39 +1099,39 @@
         <v>352687</v>
       </c>
       <c r="C2">
-        <f t="shared" ref="C2:M2" si="1">MAX(C5:C55)</f>
+        <f t="shared" ref="C2:M2" si="2">MAX(C5:C55)</f>
         <v>71</v>
       </c>
       <c r="D2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.72599999999999998</v>
       </c>
       <c r="E2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.83899999999999997</v>
       </c>
       <c r="F2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="G2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-4.0720000000000001</v>
       </c>
       <c r="H2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.10299999999999999</v>
       </c>
       <c r="I2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.94199999999999995</v>
       </c>
       <c r="J2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6.0199999999999997E-2</v>
       </c>
       <c r="K2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.73899999999999999</v>
       </c>
       <c r="L2">
@@ -1027,11 +1139,65 @@
         <v>0.72499999999999998</v>
       </c>
       <c r="M2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>184.21199999999999</v>
       </c>
+      <c r="O2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <f>MAX(P5:P55)</f>
+        <v>1</v>
+      </c>
+      <c r="Q2">
+        <f t="shared" ref="Q2:AA2" si="3">MAX(Q5:Q55)</f>
+        <v>1</v>
+      </c>
+      <c r="R2">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S2">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="T2">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="U2">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="V2">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="W2">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="X2">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="Y2">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="Z2">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="AA2">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>2</v>
       </c>
@@ -1068,8 +1234,59 @@
       <c r="M4" t="s">
         <v>13</v>
       </c>
+      <c r="P4" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>3</v>
+      </c>
+      <c r="R4" t="s">
+        <v>4</v>
+      </c>
+      <c r="S4" t="s">
+        <v>5</v>
+      </c>
+      <c r="T4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V4" t="s">
+        <v>8</v>
+      </c>
+      <c r="W4" t="s">
+        <v>9</v>
+      </c>
+      <c r="X4" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>13</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>18</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>21</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>265306</v>
       </c>
@@ -1106,8 +1323,100 @@
       <c r="M5">
         <v>82.766999999999996</v>
       </c>
+      <c r="P5">
+        <f>(B5 - $B$1)/($B$2 - $B$1)</f>
+        <v>0.58359662039485916</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" ref="Q5:Q36" si="4">(C5 - $C$1)/($C$2 - $C$1)</f>
+        <v>0.64516129032258063</v>
+      </c>
+      <c r="R5">
+        <f t="shared" ref="R5:R36" si="5">(D5 - $D$1)/($D$2 - $D$1)</f>
+        <v>0.44081632653061231</v>
+      </c>
+      <c r="S5">
+        <f t="shared" ref="S5:S36" si="6">(E5 - $E$1)/($E$2- $E$1)</f>
+        <v>0.32903565320352585</v>
+      </c>
+      <c r="T5">
+        <f t="shared" ref="T5:T36" si="7">(F5 - $F$1)/($F$2- $F$1)</f>
+        <v>0.72727272727272729</v>
+      </c>
+      <c r="U5">
+        <f t="shared" ref="U5:U36" si="8">(G5 - $G$1)/($G$2- $G$1)</f>
+        <v>0.16196046793061716</v>
+      </c>
+      <c r="V5">
+        <f t="shared" ref="V5:V36" si="9">(H5 - $H$1)/($H$2- $H$1)</f>
+        <v>0.2183462532299742</v>
+      </c>
+      <c r="W5">
+        <f t="shared" ref="W5:W36" si="10">(I5 - $I$1)/($I$2- $I$1)</f>
+        <v>1</v>
+      </c>
+      <c r="X5">
+        <f t="shared" ref="X5:X36" si="11">(J5 - $J$1)/($J$2- $J$1)</f>
+        <v>2.1262458471760802E-2</v>
+      </c>
+      <c r="Y5">
+        <f t="shared" ref="Y5:Y36" si="12">(K5 - $K$1)/($K$2- $K$1)</f>
+        <v>7.6756912442396311E-2</v>
+      </c>
+      <c r="Z5">
+        <f t="shared" ref="Z5:Z36" si="13">(L5 - $L$1)/($L$2- $L$1)</f>
+        <v>0.1569348904175332</v>
+      </c>
+      <c r="AA5">
+        <f t="shared" ref="AA5:AA36" si="14">(M5 - $M$1)/($M$2- $M$1)</f>
+        <v>0.11914871447550075</v>
+      </c>
+      <c r="AC5">
+        <f>SQRT(
+($P$1 - P5)^2 +
+($Q$1 -Q5)^2 +
+($R$1 - R5)^2 +
+($S$1 - S5)^2 +
+($T$1 - T5)^2 +
+($U$1 - U5)^2 +
+($V$1 - V5)^2 +
+($W$1 - W5)^2 +
+($X$1 - X5)^2 +
+($Y$1 - Y5)^2 +
+($Z$1 - Z5)^2 +
+($AA$1 - AA5)^2)</f>
+        <v>1.645418546063</v>
+      </c>
+      <c r="AD5">
+        <f>SQRT(
+($P$2 - P5)^2 +
+($Q$2 -Q5)^2 +
+($R$2 - R5)^2 +
+($S$2 - S5)^2 +
+($T$2 - T5)^2 +
+($U$2 - U5)^2 +
+($V$2 - V5)^2 +
+($W$2 - W5)^2 +
+($X$2 - X5)^2 +
+($Y$2 - Y5)^2 +
+($Z$2 - Z5)^2 +
+($AA$2 - AA5)^2)</f>
+        <v>2.3972520856897592</v>
+      </c>
+      <c r="AE5">
+        <f>MIN(AC5:AD5)</f>
+        <v>1.645418546063</v>
+      </c>
+      <c r="AF5">
+        <f>IF(AE5=AC5,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="AG5">
+        <f>IF(AE5=AD5,1,0)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>268653</v>
       </c>
@@ -1144,8 +1453,100 @@
       <c r="M6">
         <v>152.99700000000001</v>
       </c>
+      <c r="P6">
+        <f t="shared" ref="P6:P55" si="15">(B6 - $B$1)/($B$2 - $B$1)</f>
+        <v>0.59954633614014019</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="R6">
+        <f t="shared" si="5"/>
+        <v>0.12448979591836734</v>
+      </c>
+      <c r="S6">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="7"/>
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="U6">
+        <f t="shared" si="8"/>
+        <v>0.962081484469544</v>
+      </c>
+      <c r="V6">
+        <f t="shared" si="9"/>
+        <v>0.76485788113695097</v>
+      </c>
+      <c r="W6">
+        <f t="shared" si="10"/>
+        <v>0.42255543148827573</v>
+      </c>
+      <c r="X6">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <f t="shared" si="12"/>
+        <v>7.4740783410138248E-2</v>
+      </c>
+      <c r="Z6">
+        <f t="shared" si="13"/>
+        <v>0.32490801471764519</v>
+      </c>
+      <c r="AA6">
+        <f t="shared" si="14"/>
+        <v>0.72895881632759407</v>
+      </c>
+      <c r="AC6">
+        <f t="shared" ref="AC6:AC55" si="16">SQRT(
+($P$1 - P6)^2 +
+($Q$1 -Q6)^2 +
+($R$1 - R6)^2 +
+($S$1 - S6)^2 +
+($T$1 - T6)^2 +
+($U$1 - U6)^2 +
+($V$1 - V6)^2 +
+($W$1 - W6)^2 +
+($X$1 - X6)^2 +
+($Y$1 - Y6)^2 +
+($Z$1 - Z6)^2 +
+($AA$1 - AA6)^2)</f>
+        <v>2.2608861113651288</v>
+      </c>
+      <c r="AD6">
+        <f t="shared" ref="AD6:AD55" si="17">SQRT(
+($P$2 - P6)^2 +
+($Q$2 -Q6)^2 +
+($R$2 - R6)^2 +
+($S$2 - S6)^2 +
+($T$2 - T6)^2 +
+($U$2 - U6)^2 +
+($V$2 - V6)^2 +
+($W$2 - W6)^2 +
+($X$2 - X6)^2 +
+($Y$2 - Y6)^2 +
+($Z$2 - Z6)^2 +
+($AA$2 - AA6)^2)</f>
+        <v>1.9582138924589287</v>
+      </c>
+      <c r="AE6">
+        <f t="shared" ref="AE6:AE55" si="18">MIN(AC6:AD6)</f>
+        <v>1.9582138924589287</v>
+      </c>
+      <c r="AF6">
+        <f t="shared" ref="AF6:AF55" si="19">IF(AE6=AC6,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AG6">
+        <f t="shared" ref="AG6:AG55" si="20">IF(AE6=AD6,1,0)</f>
+        <v>1</v>
+      </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>231000</v>
       </c>
@@ -1182,8 +1583,76 @@
       <c r="M7">
         <v>172.006</v>
       </c>
+      <c r="P7">
+        <f t="shared" si="15"/>
+        <v>0.42011560803823739</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" si="4"/>
+        <v>0.90322580645161288</v>
+      </c>
+      <c r="R7">
+        <f t="shared" si="5"/>
+        <v>0.54489795918367356</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="6"/>
+        <v>0.84607288514669121</v>
+      </c>
+      <c r="T7">
+        <f t="shared" si="7"/>
+        <v>0.81818181818181823</v>
+      </c>
+      <c r="U7">
+        <f t="shared" si="8"/>
+        <v>0.64471561113352149</v>
+      </c>
+      <c r="V7">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="W7">
+        <f t="shared" si="10"/>
+        <v>0.21624926888924337</v>
+      </c>
+      <c r="X7">
+        <f t="shared" si="11"/>
+        <v>5.8471760797342194E-4</v>
+      </c>
+      <c r="Y7">
+        <f t="shared" si="12"/>
+        <v>5.7459677419354843E-2</v>
+      </c>
+      <c r="Z7">
+        <f t="shared" si="13"/>
+        <v>0.40649496080627101</v>
+      </c>
+      <c r="AA7">
+        <f t="shared" si="14"/>
+        <v>0.89401477853899125</v>
+      </c>
+      <c r="AC7">
+        <f t="shared" si="16"/>
+        <v>2.2593612109242343</v>
+      </c>
+      <c r="AD7">
+        <f t="shared" si="17"/>
+        <v>1.897547601151087</v>
+      </c>
+      <c r="AE7">
+        <f t="shared" si="18"/>
+        <v>1.897547601151087</v>
+      </c>
+      <c r="AF7">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AG7">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>238493</v>
       </c>
@@ -1220,8 +1689,76 @@
       <c r="M8">
         <v>93.620999999999995</v>
       </c>
+      <c r="P8">
+        <f t="shared" si="15"/>
+        <v>0.45582257549548005</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="4"/>
+        <v>0.83870967741935487</v>
+      </c>
+      <c r="R8">
+        <f t="shared" si="5"/>
+        <v>0.62857142857142867</v>
+      </c>
+      <c r="S8">
+        <f t="shared" si="6"/>
+        <v>0.55400605183528484</v>
+      </c>
+      <c r="T8">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="U8">
+        <f t="shared" si="8"/>
+        <v>0.57835820895522383</v>
+      </c>
+      <c r="V8">
+        <f t="shared" si="9"/>
+        <v>5.1679586563307183E-3</v>
+      </c>
+      <c r="W8">
+        <f t="shared" si="10"/>
+        <v>3.2806933588557456E-2</v>
+      </c>
+      <c r="X8">
+        <f t="shared" si="11"/>
+        <v>6.2790697674418604E-5</v>
+      </c>
+      <c r="Y8">
+        <f t="shared" si="12"/>
+        <v>9.2741935483870969E-2</v>
+      </c>
+      <c r="Z8">
+        <f t="shared" si="13"/>
+        <v>0.12334026555751078</v>
+      </c>
+      <c r="AA8">
+        <f t="shared" si="14"/>
+        <v>0.21339446195524756</v>
+      </c>
+      <c r="AC8">
+        <f t="shared" si="16"/>
+        <v>1.7372924906905118</v>
+      </c>
+      <c r="AD8">
+        <f t="shared" si="17"/>
+        <v>2.4438127223209465</v>
+      </c>
+      <c r="AE8">
+        <f t="shared" si="18"/>
+        <v>1.7372924906905118</v>
+      </c>
+      <c r="AF8">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG8">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>230098</v>
       </c>
@@ -1258,8 +1795,76 @@
       <c r="M9">
         <v>172.07499999999999</v>
       </c>
+      <c r="P9">
+        <f t="shared" si="15"/>
+        <v>0.41581723827359934</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="4"/>
+        <v>0.70967741935483875</v>
+      </c>
+      <c r="R9">
+        <f t="shared" si="5"/>
+        <v>0.67755102040816317</v>
+      </c>
+      <c r="S9">
+        <f t="shared" si="6"/>
+        <v>0.79871069596105781</v>
+      </c>
+      <c r="T9">
+        <f t="shared" si="7"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+      <c r="U9">
+        <f t="shared" si="8"/>
+        <v>0.74152884227511084</v>
+      </c>
+      <c r="V9">
+        <f t="shared" si="9"/>
+        <v>9.5607235142118871E-2</v>
+      </c>
+      <c r="W9">
+        <f t="shared" si="10"/>
+        <v>0.15776040835858987</v>
+      </c>
+      <c r="X9">
+        <f t="shared" si="11"/>
+        <v>3.0066445182724255E-5</v>
+      </c>
+      <c r="Y9">
+        <f t="shared" si="12"/>
+        <v>6.2644009216589858E-2</v>
+      </c>
+      <c r="Z9">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AA9">
+        <f t="shared" si="14"/>
+        <v>0.89461390849809408</v>
+      </c>
+      <c r="AC9">
+        <f t="shared" si="16"/>
+        <v>2.0420521714569624</v>
+      </c>
+      <c r="AD9">
+        <f t="shared" si="17"/>
+        <v>2.2091349441053221</v>
+      </c>
+      <c r="AE9">
+        <f t="shared" si="18"/>
+        <v>2.0420521714569624</v>
+      </c>
+      <c r="AF9">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG9">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>214666</v>
       </c>
@@ -1296,8 +1901,76 @@
       <c r="M10">
         <v>109.024</v>
       </c>
+      <c r="P10">
+        <f t="shared" si="15"/>
+        <v>0.34227794536019102</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" si="4"/>
+        <v>0.67741935483870963</v>
+      </c>
+      <c r="R10">
+        <f t="shared" si="5"/>
+        <v>0.66938775510204074</v>
+      </c>
+      <c r="S10">
+        <f t="shared" si="6"/>
+        <v>0.17116168925141428</v>
+      </c>
+      <c r="T10">
+        <f t="shared" si="7"/>
+        <v>0.27272727272727271</v>
+      </c>
+      <c r="U10">
+        <f t="shared" si="8"/>
+        <v>0.51089148850342869</v>
+      </c>
+      <c r="V10">
+        <f t="shared" si="9"/>
+        <v>7.8811369509043896E-2</v>
+      </c>
+      <c r="W10">
+        <f t="shared" si="10"/>
+        <v>0.76817142553304618</v>
+      </c>
+      <c r="X10">
+        <f t="shared" si="11"/>
+        <v>6.6279069767441869E-4</v>
+      </c>
+      <c r="Y10">
+        <f t="shared" si="12"/>
+        <v>8.9861751152073732E-2</v>
+      </c>
+      <c r="Z10">
+        <f t="shared" si="13"/>
+        <v>0.48328267477203651</v>
+      </c>
+      <c r="AA10">
+        <f t="shared" si="14"/>
+        <v>0.34713937152135599</v>
+      </c>
+      <c r="AC10">
+        <f t="shared" si="16"/>
+        <v>1.5320769480116152</v>
+      </c>
+      <c r="AD10">
+        <f t="shared" si="17"/>
+        <v>2.3502489222829164</v>
+      </c>
+      <c r="AE10">
+        <f t="shared" si="18"/>
+        <v>1.5320769480116152</v>
+      </c>
+      <c r="AF10">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG10">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>209906</v>
       </c>
@@ -1334,8 +2007,88 @@
       <c r="M11">
         <v>132.06200000000001</v>
       </c>
+      <c r="P11">
+        <f t="shared" si="15"/>
+        <v>0.31959475236720086</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" si="4"/>
+        <v>0.58064516129032262</v>
+      </c>
+      <c r="R11">
+        <f t="shared" si="5"/>
+        <v>0.65918367346938789</v>
+      </c>
+      <c r="S11">
+        <f t="shared" si="6"/>
+        <v>0.63557426654387594</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="U11">
+        <f t="shared" si="8"/>
+        <v>0.83844292053247271</v>
+      </c>
+      <c r="V11">
+        <f t="shared" si="9"/>
+        <v>8.9147286821705432E-2</v>
+      </c>
+      <c r="W11">
+        <f t="shared" si="10"/>
+        <v>0.21412240123358325</v>
+      </c>
+      <c r="X11">
+        <f t="shared" si="11"/>
+        <v>1.5747508305647844E-4</v>
+      </c>
+      <c r="Y11">
+        <f t="shared" si="12"/>
+        <v>0.18058755760368664</v>
+      </c>
+      <c r="Z11">
+        <f t="shared" si="13"/>
+        <v>0.52487601983682608</v>
+      </c>
+      <c r="AA11">
+        <f t="shared" si="14"/>
+        <v>0.54717931351862958</v>
+      </c>
+      <c r="AC11">
+        <f>SQRT(
+($P$1 - P11)^2 +
+($Q$1 -Q11)^2 +
+($R$1 - R11)^2 +
+($S$1 - S11)^2 +
+($T$1 - T11)^2 +
+($U$1 - U11)^2 +
+($V$1 - V11)^2 +
+($W$1 - W11)^2 +
+($X$1 - X11)^2 +
+($Y$1 - Y11)^2 +
+($Z$1 - Z11)^2 +
+($AA$1 - AA11)^2)</f>
+        <v>1.9084185791599186</v>
+      </c>
+      <c r="AD11">
+        <f t="shared" si="17"/>
+        <v>2.1125907830626516</v>
+      </c>
+      <c r="AE11">
+        <f t="shared" si="18"/>
+        <v>1.9084185791599186</v>
+      </c>
+      <c r="AF11">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG11">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>279373</v>
       </c>
@@ -1372,8 +2125,76 @@
       <c r="M12">
         <v>75.367000000000004</v>
       </c>
+      <c r="P12">
+        <f t="shared" si="15"/>
+        <v>0.65063117414116001</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" si="4"/>
+        <v>0.58064516129032262</v>
+      </c>
+      <c r="R12">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <f t="shared" si="6"/>
+        <v>0.65662412840415729</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="7"/>
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="U12">
+        <f t="shared" si="8"/>
+        <v>0.85830980233965293</v>
+      </c>
+      <c r="V12">
+        <f t="shared" si="9"/>
+        <v>0.19121447028423769</v>
+      </c>
+      <c r="W12">
+        <f t="shared" si="10"/>
+        <v>0.34598819588451113</v>
+      </c>
+      <c r="X12">
+        <f t="shared" si="11"/>
+        <v>2.4916943521594683E-3</v>
+      </c>
+      <c r="Y12">
+        <f t="shared" si="12"/>
+        <v>0.23243087557603684</v>
+      </c>
+      <c r="Z12">
+        <f t="shared" si="13"/>
+        <v>0.20332746760518317</v>
+      </c>
+      <c r="AA12">
+        <f t="shared" si="14"/>
+        <v>5.489419712243962E-2</v>
+      </c>
+      <c r="AC12">
+        <f t="shared" si="16"/>
+        <v>1.6087062896423061</v>
+      </c>
+      <c r="AD12">
+        <f t="shared" si="17"/>
+        <v>2.4004362769312833</v>
+      </c>
+      <c r="AE12">
+        <f t="shared" si="18"/>
+        <v>1.6087062896423061</v>
+      </c>
+      <c r="AF12">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG12">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>206267</v>
       </c>
@@ -1410,8 +2231,76 @@
       <c r="M13">
         <v>91.626000000000005</v>
       </c>
+      <c r="P13">
+        <f t="shared" si="15"/>
+        <v>0.30225354663159348</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="4"/>
+        <v>0.58064516129032262</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="5"/>
+        <v>0.75510204081632648</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="6"/>
+        <v>0.32508880410472307</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="7"/>
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="U13">
+        <f t="shared" si="8"/>
+        <v>0.39905203711173848</v>
+      </c>
+      <c r="V13">
+        <f t="shared" si="9"/>
+        <v>4.9095607235142093E-2</v>
+      </c>
+      <c r="W13">
+        <f t="shared" si="10"/>
+        <v>0.8925931833891636</v>
+      </c>
+      <c r="X13">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="Y13">
+        <f t="shared" si="12"/>
+        <v>0.13594470046082952</v>
+      </c>
+      <c r="Z13">
+        <f t="shared" si="13"/>
+        <v>0.50247960326347785</v>
+      </c>
+      <c r="AA13">
+        <f t="shared" si="14"/>
+        <v>0.19607179139857778</v>
+      </c>
+      <c r="AC13">
+        <f t="shared" si="16"/>
+        <v>1.7884631592625184</v>
+      </c>
+      <c r="AD13">
+        <f t="shared" si="17"/>
+        <v>2.2591515448180228</v>
+      </c>
+      <c r="AE13">
+        <f t="shared" si="18"/>
+        <v>1.7884631592625184</v>
+      </c>
+      <c r="AF13">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG13">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B14">
         <v>152946</v>
       </c>
@@ -1448,8 +2337,76 @@
       <c r="M14">
         <v>100.105</v>
       </c>
+      <c r="P14">
+        <f t="shared" si="15"/>
+        <v>4.8158896719991233E-2</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" si="4"/>
+        <v>0.41935483870967744</v>
+      </c>
+      <c r="R14">
+        <f t="shared" si="5"/>
+        <v>0.82040816326530619</v>
+      </c>
+      <c r="S14">
+        <f t="shared" si="6"/>
+        <v>0.49085646625444018</v>
+      </c>
+      <c r="T14">
+        <f t="shared" si="7"/>
+        <v>0.81818181818181823</v>
+      </c>
+      <c r="U14">
+        <f t="shared" si="8"/>
+        <v>0.44090359015732145</v>
+      </c>
+      <c r="V14">
+        <f t="shared" si="9"/>
+        <v>5.2971576227390176E-2</v>
+      </c>
+      <c r="W14">
+        <f t="shared" si="10"/>
+        <v>0.6448131015047589</v>
+      </c>
+      <c r="X14">
+        <f t="shared" si="11"/>
+        <v>0.95847176079734231</v>
+      </c>
+      <c r="Y14">
+        <f t="shared" si="12"/>
+        <v>9.7062211981566823E-2</v>
+      </c>
+      <c r="Z14">
+        <f t="shared" si="13"/>
+        <v>0.38569828827387626</v>
+      </c>
+      <c r="AA14">
+        <f t="shared" si="14"/>
+        <v>0.26969531202514613</v>
+      </c>
+      <c r="AC14">
+        <f t="shared" si="16"/>
+        <v>1.8772806642114623</v>
+      </c>
+      <c r="AD14">
+        <f t="shared" si="17"/>
+        <v>2.1519829562580086</v>
+      </c>
+      <c r="AE14">
+        <f t="shared" si="18"/>
+        <v>1.8772806642114623</v>
+      </c>
+      <c r="AF14">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG14">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B15">
         <v>212480</v>
       </c>
@@ -1486,8 +2443,76 @@
       <c r="M15">
         <v>95.597999999999999</v>
       </c>
+      <c r="P15">
+        <f t="shared" si="15"/>
+        <v>0.33186083193946064</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" si="4"/>
+        <v>0.54838709677419351</v>
+      </c>
+      <c r="R15">
+        <f t="shared" si="5"/>
+        <v>0.64897959183673481</v>
+      </c>
+      <c r="S15">
+        <f t="shared" si="6"/>
+        <v>0.51453756084725699</v>
+      </c>
+      <c r="T15">
+        <f t="shared" si="7"/>
+        <v>0.72727272727272729</v>
+      </c>
+      <c r="U15">
+        <f t="shared" si="8"/>
+        <v>0.744655102864058</v>
+      </c>
+      <c r="V15">
+        <f t="shared" si="9"/>
+        <v>0.37726098191214474</v>
+      </c>
+      <c r="W15">
+        <f t="shared" si="10"/>
+        <v>0.81708938161322919</v>
+      </c>
+      <c r="X15">
+        <f t="shared" si="11"/>
+        <v>4.3189368770764125E-5</v>
+      </c>
+      <c r="Y15">
+        <f t="shared" si="12"/>
+        <v>8.8421658986175114E-2</v>
+      </c>
+      <c r="Z15">
+        <f t="shared" si="13"/>
+        <v>0.39369700847864342</v>
+      </c>
+      <c r="AA15">
+        <f t="shared" si="14"/>
+        <v>0.2305608377399776</v>
+      </c>
+      <c r="AC15">
+        <f t="shared" si="16"/>
+        <v>1.7905739878400384</v>
+      </c>
+      <c r="AD15">
+        <f t="shared" si="17"/>
+        <v>2.0882105417468408</v>
+      </c>
+      <c r="AE15">
+        <f t="shared" si="18"/>
+        <v>1.7905739878400384</v>
+      </c>
+      <c r="AF15">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG15">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16">
         <v>241146</v>
       </c>
@@ -1524,8 +2549,76 @@
       <c r="M16">
         <v>85.471000000000004</v>
       </c>
+      <c r="P16">
+        <f t="shared" si="15"/>
+        <v>0.46846511982539663</v>
+      </c>
+      <c r="Q16">
+        <f t="shared" si="4"/>
+        <v>0.45161290322580644</v>
+      </c>
+      <c r="R16">
+        <f t="shared" si="5"/>
+        <v>0.69591836734693868</v>
+      </c>
+      <c r="S16">
+        <f t="shared" si="6"/>
+        <v>0.5934745428233128</v>
+      </c>
+      <c r="T16">
+        <f t="shared" si="7"/>
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="U16">
+        <f t="shared" si="8"/>
+        <v>0.73003227107704716</v>
+      </c>
+      <c r="V16">
+        <f t="shared" si="9"/>
+        <v>7.2351421188630458E-2</v>
+      </c>
+      <c r="W16">
+        <f t="shared" si="10"/>
+        <v>0.57675333652363492</v>
+      </c>
+      <c r="X16">
+        <f t="shared" si="11"/>
+        <v>5.4651162790697672E-5</v>
+      </c>
+      <c r="Y16">
+        <f t="shared" si="12"/>
+        <v>8.4101382488479245E-2</v>
+      </c>
+      <c r="Z16">
+        <f t="shared" si="13"/>
+        <v>0.19212925931850905</v>
+      </c>
+      <c r="AA16">
+        <f t="shared" si="14"/>
+        <v>0.14262766243802483</v>
+      </c>
+      <c r="AC16">
+        <f t="shared" si="16"/>
+        <v>1.6124647194851403</v>
+      </c>
+      <c r="AD16">
+        <f t="shared" si="17"/>
+        <v>2.304836949551937</v>
+      </c>
+      <c r="AE16">
+        <f t="shared" si="18"/>
+        <v>1.6124647194851403</v>
+      </c>
+      <c r="AF16">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG16">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B17">
         <v>185228</v>
       </c>
@@ -1562,8 +2655,76 @@
       <c r="M17">
         <v>121.69499999999999</v>
       </c>
+      <c r="P17">
+        <f t="shared" si="15"/>
+        <v>0.20199478667791296</v>
+      </c>
+      <c r="Q17">
+        <f t="shared" si="4"/>
+        <v>0.41935483870967744</v>
+      </c>
+      <c r="R17">
+        <f t="shared" si="5"/>
+        <v>0.37346938775510202</v>
+      </c>
+      <c r="S17">
+        <f t="shared" si="6"/>
+        <v>0.25009867122747009</v>
+      </c>
+      <c r="T17">
+        <f t="shared" si="7"/>
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="U17">
+        <f t="shared" si="8"/>
+        <v>0.46389673255344893</v>
+      </c>
+      <c r="V17">
+        <f t="shared" si="9"/>
+        <v>0.12919896640826872</v>
+      </c>
+      <c r="W17">
+        <f t="shared" si="10"/>
+        <v>0.66395491040569998</v>
+      </c>
+      <c r="X17">
+        <f t="shared" si="11"/>
+        <v>3.0398671096345517E-4</v>
+      </c>
+      <c r="Y17">
+        <f t="shared" si="12"/>
+        <v>0.1028225806451613</v>
+      </c>
+      <c r="Z17">
+        <f t="shared" si="13"/>
+        <v>8.3346664533674605E-2</v>
+      </c>
+      <c r="AA17">
+        <f t="shared" si="14"/>
+        <v>0.45716220792414491</v>
+      </c>
+      <c r="AC17">
+        <f t="shared" si="16"/>
+        <v>1.3125901805240408</v>
+      </c>
+      <c r="AD17">
+        <f t="shared" si="17"/>
+        <v>2.4817248522303617</v>
+      </c>
+      <c r="AE17">
+        <f t="shared" si="18"/>
+        <v>1.3125901805240408</v>
+      </c>
+      <c r="AF17">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG17">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B18">
         <v>259558</v>
       </c>
@@ -1600,8 +2761,76 @@
       <c r="M18">
         <v>139.05600000000001</v>
       </c>
+      <c r="P18">
+        <f t="shared" si="15"/>
+        <v>0.55620523524281973</v>
+      </c>
+      <c r="Q18">
+        <f t="shared" si="4"/>
+        <v>0.4838709677419355</v>
+      </c>
+      <c r="R18">
+        <f t="shared" si="5"/>
+        <v>0.24081632653061225</v>
+      </c>
+      <c r="S18">
+        <f t="shared" si="6"/>
+        <v>0.16721484015261148</v>
+      </c>
+      <c r="T18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <f t="shared" si="8"/>
+        <v>0.22075433642597822</v>
+      </c>
+      <c r="V18">
+        <f t="shared" si="9"/>
+        <v>0.14082687338501287</v>
+      </c>
+      <c r="W18">
+        <f t="shared" si="10"/>
+        <v>0.82666028606369979</v>
+      </c>
+      <c r="X18">
+        <f t="shared" si="11"/>
+        <v>3.4883720930232562E-3</v>
+      </c>
+      <c r="Y18">
+        <f t="shared" si="12"/>
+        <v>7.3876728110599074E-2</v>
+      </c>
+      <c r="Z18">
+        <f t="shared" si="13"/>
+        <v>0.16333386658134699</v>
+      </c>
+      <c r="AA18">
+        <f t="shared" si="14"/>
+        <v>0.60790851546015801</v>
+      </c>
+      <c r="AC18">
+        <f t="shared" si="16"/>
+        <v>1.3353206550251377</v>
+      </c>
+      <c r="AD18">
+        <f t="shared" si="17"/>
+        <v>2.6102046962185113</v>
+      </c>
+      <c r="AE18">
+        <f t="shared" si="18"/>
+        <v>1.3353206550251377</v>
+      </c>
+      <c r="AF18">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG18">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B19">
         <v>185421</v>
       </c>
@@ -1638,8 +2867,76 @@
       <c r="M19">
         <v>76.778999999999996</v>
       </c>
+      <c r="P19">
+        <f t="shared" si="15"/>
+        <v>0.20291450437699848</v>
+      </c>
+      <c r="Q19">
+        <f t="shared" si="4"/>
+        <v>0.38709677419354838</v>
+      </c>
+      <c r="R19">
+        <f t="shared" si="5"/>
+        <v>0.18571428571428578</v>
+      </c>
+      <c r="S19">
+        <f t="shared" si="6"/>
+        <v>0.11722141823444285</v>
+      </c>
+      <c r="T19">
+        <f t="shared" si="7"/>
+        <v>0.81818181818181823</v>
+      </c>
+      <c r="U19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="V19">
+        <f t="shared" si="9"/>
+        <v>0.31395348837209303</v>
+      </c>
+      <c r="W19">
+        <f t="shared" si="10"/>
+        <v>0.96809698516509823</v>
+      </c>
+      <c r="X19">
+        <f t="shared" si="11"/>
+        <v>0.40697674418604657</v>
+      </c>
+      <c r="Y19">
+        <f t="shared" si="12"/>
+        <v>7.5892857142857137E-2</v>
+      </c>
+      <c r="Z19">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="AA19">
+        <f t="shared" si="14"/>
+        <v>6.7154653676834472E-2</v>
+      </c>
+      <c r="AC19">
+        <f t="shared" si="16"/>
+        <v>1.4561416353579675</v>
+      </c>
+      <c r="AD19">
+        <f t="shared" si="17"/>
+        <v>2.6521578768495151</v>
+      </c>
+      <c r="AE19">
+        <f t="shared" si="18"/>
+        <v>1.4561416353579675</v>
+      </c>
+      <c r="AF19">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG19">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B20">
         <v>211674</v>
       </c>
@@ -1676,8 +2973,76 @@
       <c r="M20">
         <v>162.761</v>
       </c>
+      <c r="P20">
+        <f t="shared" si="15"/>
+        <v>0.32801993833602577</v>
+      </c>
+      <c r="Q20">
+        <f t="shared" si="4"/>
+        <v>0.35483870967741937</v>
+      </c>
+      <c r="R20">
+        <f t="shared" si="5"/>
+        <v>0.38571428571428573</v>
+      </c>
+      <c r="S20">
+        <f t="shared" si="6"/>
+        <v>0.23562689119852653</v>
+      </c>
+      <c r="T20">
+        <f t="shared" si="7"/>
+        <v>0.54545454545454541</v>
+      </c>
+      <c r="U20">
+        <f t="shared" si="8"/>
+        <v>0.47035094796288823</v>
+      </c>
+      <c r="V20">
+        <f t="shared" si="9"/>
+        <v>0.13436692506459944</v>
+      </c>
+      <c r="W20">
+        <f t="shared" si="10"/>
+        <v>0.78093263146700698</v>
+      </c>
+      <c r="X20">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="Y20">
+        <f t="shared" si="12"/>
+        <v>4.1474654377880192E-2</v>
+      </c>
+      <c r="Z20">
+        <f t="shared" si="13"/>
+        <v>0.33770596704527278</v>
+      </c>
+      <c r="AA20">
+        <f t="shared" si="14"/>
+        <v>0.81374004706209246</v>
+      </c>
+      <c r="AC20">
+        <f t="shared" si="16"/>
+        <v>1.5370108601001315</v>
+      </c>
+      <c r="AD20">
+        <f t="shared" si="17"/>
+        <v>2.3464763577212238</v>
+      </c>
+      <c r="AE20">
+        <f t="shared" si="18"/>
+        <v>1.5370108601001315</v>
+      </c>
+      <c r="AF20">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG20">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B21">
         <v>196973</v>
       </c>
@@ -1714,8 +3079,76 @@
       <c r="M21">
         <v>98.039000000000001</v>
       </c>
+      <c r="P21">
+        <f t="shared" si="15"/>
+        <v>0.25796413577511235</v>
+      </c>
+      <c r="Q21">
+        <f t="shared" si="4"/>
+        <v>0.38709677419354838</v>
+      </c>
+      <c r="R21">
+        <f t="shared" si="5"/>
+        <v>0.6673469387755101</v>
+      </c>
+      <c r="S21">
+        <f t="shared" si="6"/>
+        <v>0.5053282462833838</v>
+      </c>
+      <c r="T21">
+        <f t="shared" si="7"/>
+        <v>0.72727272727272729</v>
+      </c>
+      <c r="U21">
+        <f t="shared" si="8"/>
+        <v>0.6678096006454215</v>
+      </c>
+      <c r="V21">
+        <f t="shared" si="9"/>
+        <v>0.38113695090439281</v>
+      </c>
+      <c r="W21">
+        <f t="shared" si="10"/>
+        <v>0.85324613175945141</v>
+      </c>
+      <c r="X21">
+        <f t="shared" si="11"/>
+        <v>3.7707641196013287E-5</v>
+      </c>
+      <c r="Y21">
+        <f t="shared" si="12"/>
+        <v>6.8260368663594459E-2</v>
+      </c>
+      <c r="Z21">
+        <f t="shared" si="13"/>
+        <v>0.47048472244440892</v>
+      </c>
+      <c r="AA21">
+        <f t="shared" si="14"/>
+        <v>0.25175614542360225</v>
+      </c>
+      <c r="AC21">
+        <f t="shared" si="16"/>
+        <v>1.7477654621093495</v>
+      </c>
+      <c r="AD21">
+        <f t="shared" si="17"/>
+        <v>2.1399072902762888</v>
+      </c>
+      <c r="AE21">
+        <f t="shared" si="18"/>
+        <v>1.7477654621093495</v>
+      </c>
+      <c r="AF21">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG21">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B22">
         <v>352687</v>
       </c>
@@ -1752,8 +3185,76 @@
       <c r="M22">
         <v>156.17500000000001</v>
       </c>
+      <c r="P22">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="Q22">
+        <f t="shared" si="4"/>
+        <v>0.64516129032258063</v>
+      </c>
+      <c r="R22">
+        <f t="shared" si="5"/>
+        <v>0.30816326530612248</v>
+      </c>
+      <c r="S22">
+        <f t="shared" si="6"/>
+        <v>0.44349427706880667</v>
+      </c>
+      <c r="T22">
+        <f t="shared" si="7"/>
+        <v>0.81818181818181823</v>
+      </c>
+      <c r="U22">
+        <f t="shared" si="8"/>
+        <v>0.39209358612343687</v>
+      </c>
+      <c r="V22">
+        <f t="shared" si="9"/>
+        <v>8.3979328165374623E-2</v>
+      </c>
+      <c r="W22">
+        <f t="shared" si="10"/>
+        <v>0.91492529377359499</v>
+      </c>
+      <c r="X22">
+        <f t="shared" si="11"/>
+        <v>1.4750830564784053E-4</v>
+      </c>
+      <c r="Y22">
+        <f t="shared" si="12"/>
+        <v>0.10570276497695852</v>
+      </c>
+      <c r="Z22">
+        <f t="shared" si="13"/>
+        <v>0.24972004479283319</v>
+      </c>
+      <c r="AA22">
+        <f t="shared" si="14"/>
+        <v>0.75655352661786812</v>
+      </c>
+      <c r="AC22">
+        <f t="shared" si="16"/>
+        <v>2.0052658144813633</v>
+      </c>
+      <c r="AD22">
+        <f t="shared" si="17"/>
+        <v>2.1412252519194519</v>
+      </c>
+      <c r="AE22">
+        <f t="shared" si="18"/>
+        <v>2.0052658144813633</v>
+      </c>
+      <c r="AF22">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG22">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B23">
         <v>213732</v>
       </c>
@@ -1790,8 +3291,76 @@
       <c r="M23">
         <v>98.384</v>
       </c>
+      <c r="P23">
+        <f t="shared" si="15"/>
+        <v>0.33782708354181856</v>
+      </c>
+      <c r="Q23">
+        <f t="shared" si="4"/>
+        <v>0.61290322580645162</v>
+      </c>
+      <c r="R23">
+        <f t="shared" si="5"/>
+        <v>0.82244897959183683</v>
+      </c>
+      <c r="S23">
+        <f t="shared" si="6"/>
+        <v>0.77239836863570588</v>
+      </c>
+      <c r="T23">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="U23">
+        <f t="shared" si="8"/>
+        <v>0.62656313029447352</v>
+      </c>
+      <c r="V23">
+        <f t="shared" si="9"/>
+        <v>0.4909560723514213</v>
+      </c>
+      <c r="W23">
+        <f t="shared" si="10"/>
+        <v>0.2864359015260276</v>
+      </c>
+      <c r="X23">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="Y23">
+        <f t="shared" si="12"/>
+        <v>9.5622119815668205E-2</v>
+      </c>
+      <c r="Z23">
+        <f t="shared" si="13"/>
+        <v>0.4352903535434331</v>
+      </c>
+      <c r="AA23">
+        <f t="shared" si="14"/>
+        <v>0.25475179521911662</v>
+      </c>
+      <c r="AC23">
+        <f t="shared" si="16"/>
+        <v>1.6558935872333771</v>
+      </c>
+      <c r="AD23">
+        <f t="shared" si="17"/>
+        <v>2.2959942316105058</v>
+      </c>
+      <c r="AE23">
+        <f t="shared" si="18"/>
+        <v>1.6558935872333771</v>
+      </c>
+      <c r="AF23">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG23">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B24">
         <v>178320</v>
       </c>
@@ -1828,8 +3397,76 @@
       <c r="M24">
         <v>79.168000000000006</v>
       </c>
+      <c r="P24">
+        <f t="shared" si="15"/>
+        <v>0.16907556457800207</v>
+      </c>
+      <c r="Q24">
+        <f t="shared" si="4"/>
+        <v>0.29032258064516131</v>
+      </c>
+      <c r="R24">
+        <f t="shared" si="5"/>
+        <v>0.63061224489795931</v>
+      </c>
+      <c r="S24">
+        <f t="shared" si="6"/>
+        <v>0.35534798052887778</v>
+      </c>
+      <c r="T24">
+        <f t="shared" si="7"/>
+        <v>0.18181818181818182</v>
+      </c>
+      <c r="U24">
+        <f t="shared" si="8"/>
+        <v>0.40913674868898753</v>
+      </c>
+      <c r="V24">
+        <f t="shared" si="9"/>
+        <v>0.2868217054263566</v>
+      </c>
+      <c r="W24">
+        <f t="shared" si="10"/>
+        <v>0.50975700537034085</v>
+      </c>
+      <c r="X24">
+        <f t="shared" si="11"/>
+        <v>1E-3</v>
+      </c>
+      <c r="Y24">
+        <f t="shared" si="12"/>
+        <v>7.7620967741935484E-2</v>
+      </c>
+      <c r="Z24">
+        <f t="shared" si="13"/>
+        <v>0.39529675251959684</v>
+      </c>
+      <c r="AA24">
+        <f t="shared" si="14"/>
+        <v>8.7898443130410675E-2</v>
+      </c>
+      <c r="AC24">
+        <f t="shared" si="16"/>
+        <v>1.1616363618348051</v>
+      </c>
+      <c r="AD24">
+        <f t="shared" si="17"/>
+        <v>2.5612463150671747</v>
+      </c>
+      <c r="AE24">
+        <f t="shared" si="18"/>
+        <v>1.1616363618348051</v>
+      </c>
+      <c r="AF24">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG24">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B25">
         <v>201493</v>
       </c>
@@ -1866,8 +3503,76 @@
       <c r="M25">
         <v>87.085999999999999</v>
       </c>
+      <c r="P25">
+        <f t="shared" si="15"/>
+        <v>0.27950363836509456</v>
+      </c>
+      <c r="Q25">
+        <f t="shared" si="4"/>
+        <v>0.29032258064516131</v>
+      </c>
+      <c r="R25">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="S25">
+        <f t="shared" si="6"/>
+        <v>0.77371398500197353</v>
+      </c>
+      <c r="T25">
+        <f t="shared" si="7"/>
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="U25">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="V25">
+        <f t="shared" si="9"/>
+        <v>0.30361757105943149</v>
+      </c>
+      <c r="W25">
+        <f t="shared" si="10"/>
+        <v>0.51082043919817099</v>
+      </c>
+      <c r="X25">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="Y25">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="Z25">
+        <f t="shared" si="13"/>
+        <v>0.16813309870420731</v>
+      </c>
+      <c r="AA25">
+        <f t="shared" si="14"/>
+        <v>0.15665077669818611</v>
+      </c>
+      <c r="AC25">
+        <f t="shared" si="16"/>
+        <v>1.9983539355053765</v>
+      </c>
+      <c r="AD25">
+        <f t="shared" si="17"/>
+        <v>2.282479453143786</v>
+      </c>
+      <c r="AE25">
+        <f t="shared" si="18"/>
+        <v>1.9983539355053765</v>
+      </c>
+      <c r="AF25">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG25">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B26">
         <v>224893</v>
       </c>
@@ -1904,8 +3609,76 @@
       <c r="M26">
         <v>87.347999999999999</v>
       </c>
+      <c r="P26">
+        <f t="shared" si="15"/>
+        <v>0.3910134526583654</v>
+      </c>
+      <c r="Q26">
+        <f t="shared" si="4"/>
+        <v>0.32258064516129031</v>
+      </c>
+      <c r="R26">
+        <f t="shared" si="5"/>
+        <v>0.42448979591836739</v>
+      </c>
+      <c r="S26">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="T26">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="U26">
+        <f t="shared" si="8"/>
+        <v>1.4118596208148324E-2</v>
+      </c>
+      <c r="V26">
+        <f t="shared" si="9"/>
+        <v>0.26873385012919893</v>
+      </c>
+      <c r="W26">
+        <f t="shared" si="10"/>
+        <v>0.89152974956133357</v>
+      </c>
+      <c r="X26">
+        <f t="shared" si="11"/>
+        <v>2.7242524916943523E-3</v>
+      </c>
+      <c r="Y26">
+        <f t="shared" si="12"/>
+        <v>8.8421658986175114E-2</v>
+      </c>
+      <c r="Z26">
+        <f t="shared" si="13"/>
+        <v>8.6546152615581504E-2</v>
+      </c>
+      <c r="AA26">
+        <f t="shared" si="14"/>
+        <v>0.1589257339341999</v>
+      </c>
+      <c r="AC26">
+        <f t="shared" si="16"/>
+        <v>1.531325350053653</v>
+      </c>
+      <c r="AD26">
+        <f t="shared" si="17"/>
+        <v>2.6545789783670464</v>
+      </c>
+      <c r="AE26">
+        <f t="shared" si="18"/>
+        <v>1.531325350053653</v>
+      </c>
+      <c r="AF26">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG26">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B27">
         <v>221813</v>
       </c>
@@ -1942,8 +3715,76 @@
       <c r="M27">
         <v>107.428</v>
       </c>
+      <c r="P27">
+        <f t="shared" si="15"/>
+        <v>0.37633609248643057</v>
+      </c>
+      <c r="Q27">
+        <f t="shared" si="4"/>
+        <v>0.29032258064516131</v>
+      </c>
+      <c r="R27">
+        <f t="shared" si="5"/>
+        <v>0.74693877551020404</v>
+      </c>
+      <c r="S27">
+        <f t="shared" si="6"/>
+        <v>0.71056439942112881</v>
+      </c>
+      <c r="T27">
+        <f t="shared" si="7"/>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="U27">
+        <f t="shared" si="8"/>
+        <v>0.5843081887858006</v>
+      </c>
+      <c r="V27">
+        <f t="shared" si="9"/>
+        <v>0.12919896640826872</v>
+      </c>
+      <c r="W27">
+        <f t="shared" si="10"/>
+        <v>8.0236082309778287E-2</v>
+      </c>
+      <c r="X27">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="Y27">
+        <f t="shared" si="12"/>
+        <v>6.3508064516129031E-2</v>
+      </c>
+      <c r="Z27">
+        <f t="shared" si="13"/>
+        <v>0.20492721164613661</v>
+      </c>
+      <c r="AA27">
+        <f t="shared" si="14"/>
+        <v>0.33328123507602003</v>
+      </c>
+      <c r="AC27">
+        <f t="shared" si="16"/>
+        <v>1.4202105495195843</v>
+      </c>
+      <c r="AD27">
+        <f t="shared" si="17"/>
+        <v>2.4634658313574587</v>
+      </c>
+      <c r="AE27">
+        <f t="shared" si="18"/>
+        <v>1.4202105495195843</v>
+      </c>
+      <c r="AF27">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG27">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B28">
         <v>207600</v>
       </c>
@@ -1980,8 +3821,76 @@
       <c r="M28">
         <v>179.44300000000001</v>
       </c>
+      <c r="P28">
+        <f t="shared" si="15"/>
+        <v>0.30860579374496655</v>
+      </c>
+      <c r="Q28">
+        <f t="shared" si="4"/>
+        <v>0.38709677419354838</v>
+      </c>
+      <c r="R28">
+        <f t="shared" si="5"/>
+        <v>0.25714285714285717</v>
+      </c>
+      <c r="S28">
+        <f t="shared" si="6"/>
+        <v>0.61057755558479154</v>
+      </c>
+      <c r="T28">
+        <f t="shared" si="7"/>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="U28">
+        <f t="shared" si="8"/>
+        <v>0.69776119402985071</v>
+      </c>
+      <c r="V28">
+        <f t="shared" si="9"/>
+        <v>0.16795865633074938</v>
+      </c>
+      <c r="W28">
+        <f t="shared" si="10"/>
+        <v>0.63630563088211833</v>
+      </c>
+      <c r="X28">
+        <f t="shared" si="11"/>
+        <v>5.4651162790697672E-3</v>
+      </c>
+      <c r="Y28">
+        <f t="shared" si="12"/>
+        <v>8.1221198156682037E-2</v>
+      </c>
+      <c r="Z28">
+        <f t="shared" si="13"/>
+        <v>0.40649496080627101</v>
+      </c>
+      <c r="AA28">
+        <f t="shared" si="14"/>
+        <v>0.95859056847881796</v>
+      </c>
+      <c r="AC28">
+        <f t="shared" si="16"/>
+        <v>1.7033340397061014</v>
+      </c>
+      <c r="AD28">
+        <f t="shared" si="17"/>
+        <v>2.2266152183238019</v>
+      </c>
+      <c r="AE28">
+        <f t="shared" si="18"/>
+        <v>1.7033340397061014</v>
+      </c>
+      <c r="AF28">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG28">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B29">
         <v>142840</v>
       </c>
@@ -2018,8 +3927,76 @@
       <c r="M29">
         <v>93.296999999999997</v>
       </c>
+      <c r="P29">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="Q29">
+        <f t="shared" si="4"/>
+        <v>0.29032258064516131</v>
+      </c>
+      <c r="R29">
+        <f t="shared" si="5"/>
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="S29">
+        <f t="shared" si="6"/>
+        <v>0.82896987238521247</v>
+      </c>
+      <c r="T29">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="U29">
+        <f t="shared" si="8"/>
+        <v>0.88221056877773285</v>
+      </c>
+      <c r="V29">
+        <f t="shared" si="9"/>
+        <v>0.37596899224806202</v>
+      </c>
+      <c r="W29">
+        <f t="shared" si="10"/>
+        <v>0.29813367363215826</v>
+      </c>
+      <c r="X29">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="Y29">
+        <f t="shared" si="12"/>
+        <v>0.17338709677419356</v>
+      </c>
+      <c r="Z29">
+        <f t="shared" si="13"/>
+        <v>0.56167013277875544</v>
+      </c>
+      <c r="AA29">
+        <f t="shared" si="14"/>
+        <v>0.21058115606032976</v>
+      </c>
+      <c r="AC29">
+        <f t="shared" si="16"/>
+        <v>1.9183573797932514</v>
+      </c>
+      <c r="AD29">
+        <f t="shared" si="17"/>
+        <v>2.2380874561626469</v>
+      </c>
+      <c r="AE29">
+        <f t="shared" si="18"/>
+        <v>1.9183573797932514</v>
+      </c>
+      <c r="AF29">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG29">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B30">
         <v>270426</v>
       </c>
@@ -2056,8 +4033,76 @@
       <c r="M30">
         <v>139.785</v>
       </c>
+      <c r="P30">
+        <f t="shared" si="15"/>
+        <v>0.60799534899236107</v>
+      </c>
+      <c r="Q30">
+        <f t="shared" si="4"/>
+        <v>0.22580645161290322</v>
+      </c>
+      <c r="R30">
+        <f t="shared" si="5"/>
+        <v>0.65714285714285725</v>
+      </c>
+      <c r="S30">
+        <f t="shared" si="6"/>
+        <v>0.41981318247599009</v>
+      </c>
+      <c r="T30">
+        <f t="shared" si="7"/>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="U30">
+        <f t="shared" si="8"/>
+        <v>0.64431222267043153</v>
+      </c>
+      <c r="V30">
+        <f t="shared" si="9"/>
+        <v>5.4263565891472854E-2</v>
+      </c>
+      <c r="W30">
+        <f t="shared" si="10"/>
+        <v>0.72244377093635359</v>
+      </c>
+      <c r="X30">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="Y30">
+        <f t="shared" si="12"/>
+        <v>5.9475806451612906E-2</v>
+      </c>
+      <c r="Z30">
+        <f t="shared" si="13"/>
+        <v>0.13293872980323149</v>
+      </c>
+      <c r="AA30">
+        <f t="shared" si="14"/>
+        <v>0.61423845372372299</v>
+      </c>
+      <c r="AC30">
+        <f t="shared" si="16"/>
+        <v>1.6043207421232728</v>
+      </c>
+      <c r="AD30">
+        <f t="shared" si="17"/>
+        <v>2.3211836108145745</v>
+      </c>
+      <c r="AE30">
+        <f t="shared" si="18"/>
+        <v>1.6043207421232728</v>
+      </c>
+      <c r="AF30">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG30">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B31">
         <v>303593</v>
       </c>
@@ -2094,8 +4139,76 @@
       <c r="M31">
         <v>95.257999999999996</v>
       </c>
+      <c r="P31">
+        <f t="shared" si="15"/>
+        <v>0.76604859731137442</v>
+      </c>
+      <c r="Q31">
+        <f t="shared" si="4"/>
+        <v>0.35483870967741937</v>
+      </c>
+      <c r="R31">
+        <f t="shared" si="5"/>
+        <v>0.42448979591836739</v>
+      </c>
+      <c r="S31">
+        <f t="shared" si="6"/>
+        <v>0.85528219971056441</v>
+      </c>
+      <c r="T31">
+        <f t="shared" si="7"/>
+        <v>0.18181818181818182</v>
+      </c>
+      <c r="U31">
+        <f t="shared" si="8"/>
+        <v>0.86183945139169005</v>
+      </c>
+      <c r="V31">
+        <f t="shared" si="9"/>
+        <v>3.2299741602067167E-2</v>
+      </c>
+      <c r="W31">
+        <f t="shared" si="10"/>
+        <v>5.6361992874993348E-3</v>
+      </c>
+      <c r="X31">
+        <f t="shared" si="11"/>
+        <v>2.9900332225913621E-5</v>
+      </c>
+      <c r="Y31">
+        <f t="shared" si="12"/>
+        <v>3.7010368663594473E-2</v>
+      </c>
+      <c r="Z31">
+        <f t="shared" si="13"/>
+        <v>0.46088625819868828</v>
+      </c>
+      <c r="AA31">
+        <f t="shared" si="14"/>
+        <v>0.22760860315889098</v>
+      </c>
+      <c r="AC31">
+        <f t="shared" si="16"/>
+        <v>1.633074373714976</v>
+      </c>
+      <c r="AD31">
+        <f t="shared" si="17"/>
+        <v>2.5002711644826512</v>
+      </c>
+      <c r="AE31">
+        <f t="shared" si="18"/>
+        <v>1.633074373714976</v>
+      </c>
+      <c r="AF31">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG31">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B32">
         <v>230108</v>
       </c>
@@ -2132,8 +4245,76 @@
       <c r="M32">
         <v>91.647999999999996</v>
       </c>
+      <c r="P32">
+        <f t="shared" si="15"/>
+        <v>0.41586489204039134</v>
+      </c>
+      <c r="Q32">
+        <f t="shared" si="4"/>
+        <v>0.22580645161290322</v>
+      </c>
+      <c r="R32">
+        <f t="shared" si="5"/>
+        <v>0.62448979591836751</v>
+      </c>
+      <c r="S32">
+        <f t="shared" si="6"/>
+        <v>0.66451782660176295</v>
+      </c>
+      <c r="T32">
+        <f t="shared" si="7"/>
+        <v>0.81818181818181823</v>
+      </c>
+      <c r="U32">
+        <f t="shared" si="8"/>
+        <v>0.72650262202501004</v>
+      </c>
+      <c r="V32">
+        <f t="shared" si="9"/>
+        <v>0.42764857881136958</v>
+      </c>
+      <c r="W32">
+        <f t="shared" si="10"/>
+        <v>0.40554049024299471</v>
+      </c>
+      <c r="X32">
+        <f t="shared" si="11"/>
+        <v>5.3820598006644525E-4</v>
+      </c>
+      <c r="Y32">
+        <f t="shared" si="12"/>
+        <v>0.363479262672811</v>
+      </c>
+      <c r="Z32">
+        <f t="shared" si="13"/>
+        <v>0.23532234842425215</v>
+      </c>
+      <c r="AA32">
+        <f t="shared" si="14"/>
+        <v>0.19626281834205977</v>
+      </c>
+      <c r="AC32">
+        <f t="shared" si="16"/>
+        <v>1.6810980692060249</v>
+      </c>
+      <c r="AD32">
+        <f t="shared" si="17"/>
+        <v>2.1489021607743366</v>
+      </c>
+      <c r="AE32">
+        <f t="shared" si="18"/>
+        <v>1.6810980692060249</v>
+      </c>
+      <c r="AF32">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG32">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B33">
         <v>193373</v>
       </c>
@@ -2170,8 +4351,76 @@
       <c r="M33">
         <v>119.22</v>
       </c>
+      <c r="P33">
+        <f t="shared" si="15"/>
+        <v>0.24080877972999376</v>
+      </c>
+      <c r="Q33">
+        <f t="shared" si="4"/>
+        <v>0.25806451612903225</v>
+      </c>
+      <c r="R33">
+        <f t="shared" si="5"/>
+        <v>0.42448979591836739</v>
+      </c>
+      <c r="S33">
+        <f t="shared" si="6"/>
+        <v>0.63031180107880558</v>
+      </c>
+      <c r="T33">
+        <f t="shared" si="7"/>
+        <v>0.72727272727272729</v>
+      </c>
+      <c r="U33">
+        <f t="shared" si="8"/>
+        <v>0.83743444937474765</v>
+      </c>
+      <c r="V33">
+        <f t="shared" si="9"/>
+        <v>0.1731266149870801</v>
+      </c>
+      <c r="W33">
+        <f t="shared" si="10"/>
+        <v>0.29813367363215826</v>
+      </c>
+      <c r="X33">
+        <f t="shared" si="11"/>
+        <v>2.4750830564784055E-5</v>
+      </c>
+      <c r="Y33">
+        <f t="shared" si="12"/>
+        <v>8.2661290322580627E-2</v>
+      </c>
+      <c r="Z33">
+        <f t="shared" si="13"/>
+        <v>0.2305231163013918</v>
+      </c>
+      <c r="AA33">
+        <f t="shared" si="14"/>
+        <v>0.43567167678241164</v>
+      </c>
+      <c r="AC33">
+        <f t="shared" si="16"/>
+        <v>1.5168826295836715</v>
+      </c>
+      <c r="AD33">
+        <f t="shared" si="17"/>
+        <v>2.3714734928337173</v>
+      </c>
+      <c r="AE33">
+        <f t="shared" si="18"/>
+        <v>1.5168826295836715</v>
+      </c>
+      <c r="AF33">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG33">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B34">
         <v>222293</v>
       </c>
@@ -2208,8 +4457,76 @@
       <c r="M34">
         <v>135.25700000000001</v>
       </c>
+      <c r="P34">
+        <f t="shared" si="15"/>
+        <v>0.37862347329244639</v>
+      </c>
+      <c r="Q34">
+        <f t="shared" si="4"/>
+        <v>0.22580645161290322</v>
+      </c>
+      <c r="R34">
+        <f t="shared" si="5"/>
+        <v>0.62653061224489803</v>
+      </c>
+      <c r="S34">
+        <f t="shared" si="6"/>
+        <v>0.32640442047099066</v>
+      </c>
+      <c r="T34">
+        <f t="shared" si="7"/>
+        <v>0.81818181818181823</v>
+      </c>
+      <c r="U34">
+        <f t="shared" si="8"/>
+        <v>0.72357805566760791</v>
+      </c>
+      <c r="V34">
+        <f t="shared" si="9"/>
+        <v>0.14470284237726097</v>
+      </c>
+      <c r="W34">
+        <f t="shared" si="10"/>
+        <v>0.83304088903068019</v>
+      </c>
+      <c r="X34">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="Y34">
+        <f t="shared" si="12"/>
+        <v>6.3652073732718903E-2</v>
+      </c>
+      <c r="Z34">
+        <f t="shared" si="13"/>
+        <v>0.23852183650615905</v>
+      </c>
+      <c r="AA34">
+        <f t="shared" si="14"/>
+        <v>0.57492163553795805</v>
+      </c>
+      <c r="AC34">
+        <f t="shared" si="16"/>
+        <v>1.7299672272986877</v>
+      </c>
+      <c r="AD34">
+        <f t="shared" si="17"/>
+        <v>2.2549630573950932</v>
+      </c>
+      <c r="AE34">
+        <f t="shared" si="18"/>
+        <v>1.7299672272986877</v>
+      </c>
+      <c r="AF34">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG34">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B35">
         <v>220720</v>
       </c>
@@ -2246,8 +4563,76 @@
       <c r="M35">
         <v>141.36000000000001</v>
       </c>
+      <c r="P35">
+        <f t="shared" si="15"/>
+        <v>0.37112753577606544</v>
+      </c>
+      <c r="Q35">
+        <f t="shared" si="4"/>
+        <v>0.19354838709677419</v>
+      </c>
+      <c r="R35">
+        <f t="shared" si="5"/>
+        <v>0.45102040816326538</v>
+      </c>
+      <c r="S35">
+        <f t="shared" si="6"/>
+        <v>0.37771345875542695</v>
+      </c>
+      <c r="T35">
+        <f t="shared" si="7"/>
+        <v>0.18181818181818182</v>
+      </c>
+      <c r="U35">
+        <f t="shared" si="8"/>
+        <v>0.66659943525615162</v>
+      </c>
+      <c r="V35">
+        <f t="shared" si="9"/>
+        <v>0.20284237726098195</v>
+      </c>
+      <c r="W35">
+        <f t="shared" si="10"/>
+        <v>0.84048492582549061</v>
+      </c>
+      <c r="X35">
+        <f t="shared" si="11"/>
+        <v>5.0996677740863794E-4</v>
+      </c>
+      <c r="Y35">
+        <f t="shared" si="12"/>
+        <v>6.2644009216589858E-2</v>
+      </c>
+      <c r="Z35">
+        <f t="shared" si="13"/>
+        <v>0.26091825307950733</v>
+      </c>
+      <c r="AA35">
+        <f t="shared" si="14"/>
+        <v>0.62791424626846248</v>
+      </c>
+      <c r="AC35">
+        <f t="shared" si="16"/>
+        <v>1.4874593297814147</v>
+      </c>
+      <c r="AD35">
+        <f t="shared" si="17"/>
+        <v>2.3954650669891144</v>
+      </c>
+      <c r="AE35">
+        <f t="shared" si="18"/>
+        <v>1.4874593297814147</v>
+      </c>
+      <c r="AF35">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG35">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B36">
         <v>231693</v>
       </c>
@@ -2284,8 +4669,76 @@
       <c r="M36">
         <v>167.64699999999999</v>
       </c>
+      <c r="P36">
+        <f t="shared" si="15"/>
+        <v>0.4234180140769227</v>
+      </c>
+      <c r="Q36">
+        <f t="shared" si="4"/>
+        <v>0.16129032258064516</v>
+      </c>
+      <c r="R36">
+        <f t="shared" si="5"/>
+        <v>0.37959183673469388</v>
+      </c>
+      <c r="S36">
+        <f t="shared" si="6"/>
+        <v>0.52111564267859489</v>
+      </c>
+      <c r="T36">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="U36">
+        <f t="shared" si="8"/>
+        <v>0.81070996369503823</v>
+      </c>
+      <c r="V36">
+        <f t="shared" si="9"/>
+        <v>0.1459948320413437</v>
+      </c>
+      <c r="W36">
+        <f t="shared" si="10"/>
+        <v>0.48210772584675926</v>
+      </c>
+      <c r="X36">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="Y36">
+        <f t="shared" si="12"/>
+        <v>0.14314516129032256</v>
+      </c>
+      <c r="Z36">
+        <f t="shared" si="13"/>
+        <v>0.3025115981442969</v>
+      </c>
+      <c r="AA36">
+        <f t="shared" si="14"/>
+        <v>0.85616539460088392</v>
+      </c>
+      <c r="AC36">
+        <f t="shared" si="16"/>
+        <v>1.8376519912720193</v>
+      </c>
+      <c r="AD36">
+        <f t="shared" si="17"/>
+        <v>2.2192034286308715</v>
+      </c>
+      <c r="AE36">
+        <f t="shared" si="18"/>
+        <v>1.8376519912720193</v>
+      </c>
+      <c r="AF36">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG36">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B37">
         <v>174933</v>
       </c>
@@ -2322,8 +4775,76 @@
       <c r="M37">
         <v>139.38999999999999</v>
       </c>
+      <c r="P37">
+        <f t="shared" si="15"/>
+        <v>0.15293523376555299</v>
+      </c>
+      <c r="Q37">
+        <f t="shared" ref="Q37:Q55" si="21">(C37 - $C$1)/($C$2 - $C$1)</f>
+        <v>0.29032258064516131</v>
+      </c>
+      <c r="R37">
+        <f t="shared" ref="R37:R55" si="22">(D37 - $D$1)/($D$2 - $D$1)</f>
+        <v>0.7</v>
+      </c>
+      <c r="S37">
+        <f t="shared" ref="S37:S55" si="23">(E37 - $E$1)/($E$2- $E$1)</f>
+        <v>0.71319563215366399</v>
+      </c>
+      <c r="T37">
+        <f t="shared" ref="T37:T55" si="24">(F37 - $F$1)/($F$2- $F$1)</f>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="U37">
+        <f t="shared" ref="U37:U55" si="25">(G37 - $G$1)/($G$2- $G$1)</f>
+        <v>0.81222267043162544</v>
+      </c>
+      <c r="V37">
+        <f t="shared" ref="V37:V55" si="26">(H37 - $H$1)/($H$2- $H$1)</f>
+        <v>0.12532299741602063</v>
+      </c>
+      <c r="W37">
+        <f t="shared" ref="W37:W55" si="27">(I37 - $I$1)/($I$2- $I$1)</f>
+        <v>0.28537246769819752</v>
+      </c>
+      <c r="X37">
+        <f t="shared" ref="X37:X55" si="28">(J37 - $J$1)/($J$2- $J$1)</f>
+        <v>0</v>
+      </c>
+      <c r="Y37">
+        <f t="shared" ref="Y37:Y55" si="29">(K37 - $K$1)/($K$2- $K$1)</f>
+        <v>7.4740783410138248E-2</v>
+      </c>
+      <c r="Z37">
+        <f t="shared" ref="Z37:Z55" si="30">(L37 - $L$1)/($L$2- $L$1)</f>
+        <v>0.81762917933130697</v>
+      </c>
+      <c r="AA37">
+        <f t="shared" ref="AA37:AA55" si="31">(M37 - $M$1)/($M$2- $M$1)</f>
+        <v>0.61080865178393107</v>
+      </c>
+      <c r="AC37">
+        <f t="shared" si="16"/>
+        <v>1.7654959078366099</v>
+      </c>
+      <c r="AD37">
+        <f t="shared" si="17"/>
+        <v>2.2456145034768791</v>
+      </c>
+      <c r="AE37">
+        <f t="shared" si="18"/>
+        <v>1.7654959078366099</v>
+      </c>
+      <c r="AF37">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG37">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="38" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B38">
         <v>291533</v>
       </c>
@@ -2360,8 +4881,76 @@
       <c r="M38">
         <v>152.65100000000001</v>
       </c>
+      <c r="P38">
+        <f t="shared" si="15"/>
+        <v>0.70857815456022721</v>
+      </c>
+      <c r="Q38">
+        <f t="shared" si="21"/>
+        <v>0.29032258064516131</v>
+      </c>
+      <c r="R38">
+        <f t="shared" si="22"/>
+        <v>0.3693877551020408</v>
+      </c>
+      <c r="S38">
+        <f t="shared" si="23"/>
+        <v>0.73029864491514285</v>
+      </c>
+      <c r="T38">
+        <f t="shared" si="24"/>
+        <v>0.81818181818181823</v>
+      </c>
+      <c r="U38">
+        <f t="shared" si="25"/>
+        <v>0.68646631706333194</v>
+      </c>
+      <c r="V38">
+        <f t="shared" si="26"/>
+        <v>0.29198966408268734</v>
+      </c>
+      <c r="W38">
+        <f t="shared" si="27"/>
+        <v>1.6642739405540494E-2</v>
+      </c>
+      <c r="X38">
+        <f t="shared" si="28"/>
+        <v>3.3554817275747512E-4</v>
+      </c>
+      <c r="Y38">
+        <f t="shared" si="29"/>
+        <v>9.8502304147465441E-2</v>
+      </c>
+      <c r="Z38">
+        <f t="shared" si="30"/>
+        <v>0.35370340745480727</v>
+      </c>
+      <c r="AA38">
+        <f t="shared" si="31"/>
+        <v>0.72595448348919411</v>
+      </c>
+      <c r="AC38">
+        <f t="shared" si="16"/>
+        <v>1.7731793175442365</v>
+      </c>
+      <c r="AD38">
+        <f t="shared" si="17"/>
+        <v>2.2278774781675712</v>
+      </c>
+      <c r="AE38">
+        <f t="shared" si="18"/>
+        <v>1.7731793175442365</v>
+      </c>
+      <c r="AF38">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG38">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="39" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B39">
         <v>287346</v>
       </c>
@@ -2398,8 +4987,76 @@
       <c r="M39">
         <v>128.96899999999999</v>
       </c>
+      <c r="P39">
+        <f t="shared" si="15"/>
+        <v>0.68862552240441843</v>
+      </c>
+      <c r="Q39">
+        <f t="shared" si="21"/>
+        <v>0.16129032258064516</v>
+      </c>
+      <c r="R39">
+        <f t="shared" si="22"/>
+        <v>0.6183673469387756</v>
+      </c>
+      <c r="S39">
+        <f t="shared" si="23"/>
+        <v>0.14221812919352717</v>
+      </c>
+      <c r="T39">
+        <f t="shared" si="24"/>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="U39">
+        <f t="shared" si="25"/>
+        <v>0.22509076240419515</v>
+      </c>
+      <c r="V39">
+        <f t="shared" si="26"/>
+        <v>0.12532299741602063</v>
+      </c>
+      <c r="W39">
+        <f t="shared" si="27"/>
+        <v>0.88408571276652315</v>
+      </c>
+      <c r="X39">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="Y39">
+        <f t="shared" si="29"/>
+        <v>0.10714285714285714</v>
+      </c>
+      <c r="Z39">
+        <f t="shared" si="30"/>
+        <v>0.40969444888817791</v>
+      </c>
+      <c r="AA39">
+        <f t="shared" si="31"/>
+        <v>0.52032266187362697</v>
+      </c>
+      <c r="AC39">
+        <f t="shared" si="16"/>
+        <v>1.5516054520428109</v>
+      </c>
+      <c r="AD39">
+        <f t="shared" si="17"/>
+        <v>2.3945912065529122</v>
+      </c>
+      <c r="AE39">
+        <f t="shared" si="18"/>
+        <v>1.5516054520428109</v>
+      </c>
+      <c r="AF39">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG39">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B40">
         <v>182186</v>
       </c>
@@ -2436,8 +5093,76 @@
       <c r="M40">
         <v>145.77199999999999</v>
       </c>
+      <c r="P40">
+        <f t="shared" si="15"/>
+        <v>0.18749851081978774</v>
+      </c>
+      <c r="Q40">
+        <f t="shared" si="21"/>
+        <v>0.16129032258064516</v>
+      </c>
+      <c r="R40">
+        <f t="shared" si="22"/>
+        <v>0.65510204081632673</v>
+      </c>
+      <c r="S40">
+        <f t="shared" si="23"/>
+        <v>0.13958689646099198</v>
+      </c>
+      <c r="T40">
+        <f t="shared" si="24"/>
+        <v>0.72727272727272729</v>
+      </c>
+      <c r="U40">
+        <f t="shared" si="25"/>
+        <v>0.18293666801129488</v>
+      </c>
+      <c r="V40">
+        <f t="shared" si="26"/>
+        <v>0.23643410852713179</v>
+      </c>
+      <c r="W40">
+        <f t="shared" si="27"/>
+        <v>0.96916041899292826</v>
+      </c>
+      <c r="X40">
+        <f t="shared" si="28"/>
+        <v>3.6877076411960134E-4</v>
+      </c>
+      <c r="Y40">
+        <f t="shared" si="29"/>
+        <v>0.15178571428571427</v>
+      </c>
+      <c r="Z40">
+        <f t="shared" si="30"/>
+        <v>0.50887857942729164</v>
+      </c>
+      <c r="AA40">
+        <f t="shared" si="31"/>
+        <v>0.6662238314795037</v>
+      </c>
+      <c r="AC40">
+        <f t="shared" si="16"/>
+        <v>1.6712954664878252</v>
+      </c>
+      <c r="AD40">
+        <f t="shared" si="17"/>
+        <v>2.3706858411493141</v>
+      </c>
+      <c r="AE40">
+        <f t="shared" si="18"/>
+        <v>1.6712954664878252</v>
+      </c>
+      <c r="AF40">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG40">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="41" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B41">
         <v>169920</v>
       </c>
@@ -2474,8 +5199,76 @@
       <c r="M41">
         <v>171.92</v>
       </c>
+      <c r="P41">
+        <f t="shared" si="15"/>
+        <v>0.12904640047272536</v>
+      </c>
+      <c r="Q41">
+        <f t="shared" si="21"/>
+        <v>0.19354838709677419</v>
+      </c>
+      <c r="R41">
+        <f t="shared" si="22"/>
+        <v>0.34081632653061233</v>
+      </c>
+      <c r="S41">
+        <f t="shared" si="23"/>
+        <v>0.68030522299697405</v>
+      </c>
+      <c r="T41">
+        <f t="shared" si="24"/>
+        <v>0.18181818181818182</v>
+      </c>
+      <c r="U41">
+        <f t="shared" si="25"/>
+        <v>0.73023396530859208</v>
+      </c>
+      <c r="V41">
+        <f t="shared" si="26"/>
+        <v>8.3979328165374623E-2</v>
+      </c>
+      <c r="W41">
+        <f t="shared" si="27"/>
+        <v>0.26942096028074658</v>
+      </c>
+      <c r="X41">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="Y41">
+        <f t="shared" si="29"/>
+        <v>0.37788018433179715</v>
+      </c>
+      <c r="Z41">
+        <f t="shared" si="30"/>
+        <v>0.79043353063509836</v>
+      </c>
+      <c r="AA41">
+        <f t="shared" si="31"/>
+        <v>0.893268036850834</v>
+      </c>
+      <c r="AC41">
+        <f t="shared" si="16"/>
+        <v>1.6865737395499323</v>
+      </c>
+      <c r="AD41">
+        <f t="shared" si="17"/>
+        <v>2.3458537742075958</v>
+      </c>
+      <c r="AE41">
+        <f t="shared" si="18"/>
+        <v>1.6865737395499323</v>
+      </c>
+      <c r="AF41">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG41">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="42" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B42">
         <v>156146</v>
       </c>
@@ -2512,8 +5305,76 @@
       <c r="M42">
         <v>114.142</v>
       </c>
+      <c r="P42">
+        <f t="shared" si="15"/>
+        <v>6.340810209342998E-2</v>
+      </c>
+      <c r="Q42">
+        <f t="shared" si="21"/>
+        <v>9.6774193548387094E-2</v>
+      </c>
+      <c r="R42">
+        <f t="shared" si="22"/>
+        <v>0.84489795918367361</v>
+      </c>
+      <c r="S42">
+        <f t="shared" si="23"/>
+        <v>0.14353374555979476</v>
+      </c>
+      <c r="T42">
+        <f t="shared" si="24"/>
+        <v>0.81818181818181823</v>
+      </c>
+      <c r="U42">
+        <f t="shared" si="25"/>
+        <v>0.29729729729729731</v>
+      </c>
+      <c r="V42">
+        <f t="shared" si="26"/>
+        <v>0.17571059431524547</v>
+      </c>
+      <c r="W42">
+        <f t="shared" si="27"/>
+        <v>0.93619397033019625</v>
+      </c>
+      <c r="X42">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="Y42">
+        <f t="shared" si="29"/>
+        <v>9.994239631336406E-2</v>
+      </c>
+      <c r="Z42">
+        <f t="shared" si="30"/>
+        <v>0.24652055671092629</v>
+      </c>
+      <c r="AA42">
+        <f t="shared" si="31"/>
+        <v>0.39157918500959477</v>
+      </c>
+      <c r="AC42">
+        <f t="shared" si="16"/>
+        <v>1.6239076293652632</v>
+      </c>
+      <c r="AD42">
+        <f t="shared" si="17"/>
+        <v>2.531599563837704</v>
+      </c>
+      <c r="AE42">
+        <f t="shared" si="18"/>
+        <v>1.6239076293652632</v>
+      </c>
+      <c r="AF42">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG42">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="43" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B43">
         <v>286093</v>
       </c>
@@ -2550,8 +5411,76 @@
       <c r="M43">
         <v>69.045000000000002</v>
       </c>
+      <c r="P43">
+        <f t="shared" si="15"/>
+        <v>0.68265450542538131</v>
+      </c>
+      <c r="Q43">
+        <f t="shared" si="21"/>
+        <v>0.19354838709677419</v>
+      </c>
+      <c r="R43">
+        <f t="shared" si="22"/>
+        <v>0.3836734693877551</v>
+      </c>
+      <c r="S43">
+        <f t="shared" si="23"/>
+        <v>0.23694250756479412</v>
+      </c>
+      <c r="T43">
+        <f t="shared" si="24"/>
+        <v>0.81818181818181823</v>
+      </c>
+      <c r="U43">
+        <f t="shared" si="25"/>
+        <v>4.0641387656312894E-2</v>
+      </c>
+      <c r="V43">
+        <f t="shared" si="26"/>
+        <v>0.24289405684754525</v>
+      </c>
+      <c r="W43">
+        <f t="shared" si="27"/>
+        <v>0.99361939703301971</v>
+      </c>
+      <c r="X43">
+        <f t="shared" si="28"/>
+        <v>3.4717607973421925E-5</v>
+      </c>
+      <c r="Y43">
+        <f t="shared" si="29"/>
+        <v>1</v>
+      </c>
+      <c r="Z43">
+        <f t="shared" si="30"/>
+        <v>0.6192609182530795</v>
+      </c>
+      <c r="AA43">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+      <c r="AC43">
+        <f t="shared" si="16"/>
+        <v>1.95132251563279</v>
+      </c>
+      <c r="AD43">
+        <f t="shared" si="17"/>
+        <v>2.3205079680765097</v>
+      </c>
+      <c r="AE43">
+        <f t="shared" si="18"/>
+        <v>1.95132251563279</v>
+      </c>
+      <c r="AF43">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG43">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B44">
         <v>206268</v>
       </c>
@@ -2588,8 +5517,76 @@
       <c r="M44">
         <v>118.68600000000001</v>
       </c>
+      <c r="P44">
+        <f t="shared" si="15"/>
+        <v>0.30225831200827269</v>
+      </c>
+      <c r="Q44">
+        <f t="shared" si="21"/>
+        <v>0.12903225806451613</v>
+      </c>
+      <c r="R44">
+        <f t="shared" si="22"/>
+        <v>0.92040816326530628</v>
+      </c>
+      <c r="S44">
+        <f t="shared" si="23"/>
+        <v>0.94605972898302859</v>
+      </c>
+      <c r="T44">
+        <f t="shared" si="24"/>
+        <v>0.27272727272727271</v>
+      </c>
+      <c r="U44">
+        <f t="shared" si="25"/>
+        <v>0.85114965711980628</v>
+      </c>
+      <c r="V44">
+        <f t="shared" si="26"/>
+        <v>0.49224806201550403</v>
+      </c>
+      <c r="W44">
+        <f t="shared" si="27"/>
+        <v>0.14606263625245922</v>
+      </c>
+      <c r="X44">
+        <f t="shared" si="28"/>
+        <v>3.4883720930232559E-4</v>
+      </c>
+      <c r="Y44">
+        <f t="shared" si="29"/>
+        <v>6.5092165898617521E-2</v>
+      </c>
+      <c r="Z44">
+        <f t="shared" si="30"/>
+        <v>0.92801151815709493</v>
+      </c>
+      <c r="AA44">
+        <f t="shared" si="31"/>
+        <v>0.43103493188152864</v>
+      </c>
+      <c r="AC44">
+        <f t="shared" si="16"/>
+        <v>1.9909549374766757</v>
+      </c>
+      <c r="AD44">
+        <f t="shared" si="17"/>
+        <v>2.2349573767518107</v>
+      </c>
+      <c r="AE44">
+        <f t="shared" si="18"/>
+        <v>1.9909549374766757</v>
+      </c>
+      <c r="AF44">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG44">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B45">
         <v>151333</v>
       </c>
@@ -2626,8 +5623,76 @@
       <c r="M45">
         <v>80.338999999999999</v>
       </c>
+      <c r="P45">
+        <f t="shared" si="15"/>
+        <v>4.0472344136442268E-2</v>
+      </c>
+      <c r="Q45">
+        <f t="shared" si="21"/>
+        <v>3.2258064516129031E-2</v>
+      </c>
+      <c r="R45">
+        <f t="shared" si="22"/>
+        <v>0.65102040816326545</v>
+      </c>
+      <c r="S45">
+        <f t="shared" si="23"/>
+        <v>0.38297592422049731</v>
+      </c>
+      <c r="T45">
+        <f t="shared" si="24"/>
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="U45">
+        <f t="shared" si="25"/>
+        <v>0.41962484872932626</v>
+      </c>
+      <c r="V45">
+        <f t="shared" si="26"/>
+        <v>6.2015503875968978E-2</v>
+      </c>
+      <c r="W45">
+        <f t="shared" si="27"/>
+        <v>0.90322752166746423</v>
+      </c>
+      <c r="X45">
+        <f t="shared" si="28"/>
+        <v>3.4219269102990033E-3</v>
+      </c>
+      <c r="Y45">
+        <f t="shared" si="29"/>
+        <v>0.12154377880184332</v>
+      </c>
+      <c r="Z45">
+        <f t="shared" si="30"/>
+        <v>0.69284914413693821</v>
+      </c>
+      <c r="AA45">
+        <f t="shared" si="31"/>
+        <v>9.8066286349388257E-2</v>
+      </c>
+      <c r="AC45">
+        <f t="shared" si="16"/>
+        <v>1.7028844440607467</v>
+      </c>
+      <c r="AD45">
+        <f t="shared" si="17"/>
+        <v>2.5033341983497004</v>
+      </c>
+      <c r="AE45">
+        <f t="shared" si="18"/>
+        <v>1.7028844440607467</v>
+      </c>
+      <c r="AF45">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG45">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B46">
         <v>209051</v>
       </c>
@@ -2664,8 +5729,76 @@
       <c r="M46">
         <v>172.709</v>
       </c>
+      <c r="P46">
+        <f t="shared" si="15"/>
+        <v>0.3155203553064852</v>
+      </c>
+      <c r="Q46">
+        <f t="shared" si="21"/>
+        <v>0.16129032258064516</v>
+      </c>
+      <c r="R46">
+        <f t="shared" si="22"/>
+        <v>0.36530612244897959</v>
+      </c>
+      <c r="S46">
+        <f t="shared" si="23"/>
+        <v>0.68425207209577688</v>
+      </c>
+      <c r="T46">
+        <f t="shared" si="24"/>
+        <v>0.18181818181818182</v>
+      </c>
+      <c r="U46">
+        <f t="shared" si="25"/>
+        <v>0.81655909640984259</v>
+      </c>
+      <c r="V46">
+        <f t="shared" si="26"/>
+        <v>8.0103359173126623E-2</v>
+      </c>
+      <c r="W46">
+        <f t="shared" si="27"/>
+        <v>0.23113734247886425</v>
+      </c>
+      <c r="X46">
+        <f t="shared" si="28"/>
+        <v>1.8438538205980066E-5</v>
+      </c>
+      <c r="Y46">
+        <f t="shared" si="29"/>
+        <v>0.40812211981566815</v>
+      </c>
+      <c r="Z46">
+        <f t="shared" si="30"/>
+        <v>0.72484402495600719</v>
+      </c>
+      <c r="AA46">
+        <f t="shared" si="31"/>
+        <v>0.90011895768753214</v>
+      </c>
+      <c r="AC46">
+        <f t="shared" si="16"/>
+        <v>1.7288902266977622</v>
+      </c>
+      <c r="AD46">
+        <f t="shared" si="17"/>
+        <v>2.2914800084993994</v>
+      </c>
+      <c r="AE46">
+        <f t="shared" si="18"/>
+        <v>1.7288902266977622</v>
+      </c>
+      <c r="AF46">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG46">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B47">
         <v>211600</v>
       </c>
@@ -2702,8 +5835,76 @@
       <c r="M47">
         <v>97.814999999999998</v>
       </c>
+      <c r="P47">
+        <f t="shared" si="15"/>
+        <v>0.32766730046176501</v>
+      </c>
+      <c r="Q47">
+        <f t="shared" si="21"/>
+        <v>6.4516129032258063E-2</v>
+      </c>
+      <c r="R47">
+        <f t="shared" si="22"/>
+        <v>0.67551020408163254</v>
+      </c>
+      <c r="S47">
+        <f t="shared" si="23"/>
+        <v>0.77108275226943834</v>
+      </c>
+      <c r="T47">
+        <f t="shared" si="24"/>
+        <v>1</v>
+      </c>
+      <c r="U47">
+        <f t="shared" si="25"/>
+        <v>0.96036708350141176</v>
+      </c>
+      <c r="V47">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="W47">
+        <f t="shared" si="27"/>
+        <v>7.4174509491146928E-2</v>
+      </c>
+      <c r="X47">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="Y47">
+        <f t="shared" si="29"/>
+        <v>0.19066820276497695</v>
+      </c>
+      <c r="Z47">
+        <f t="shared" si="30"/>
+        <v>0.79683250679891215</v>
+      </c>
+      <c r="AA47">
+        <f t="shared" si="31"/>
+        <v>0.24981114381723932</v>
+      </c>
+      <c r="AC47">
+        <f t="shared" si="16"/>
+        <v>1.9554845039801849</v>
+      </c>
+      <c r="AD47">
+        <f t="shared" si="17"/>
+        <v>2.3669938700531246</v>
+      </c>
+      <c r="AE47">
+        <f t="shared" si="18"/>
+        <v>1.9554845039801849</v>
+      </c>
+      <c r="AF47">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG47">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="48" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B48">
         <v>309746</v>
       </c>
@@ -2740,8 +5941,76 @@
       <c r="M48">
         <v>184.21199999999999</v>
       </c>
+      <c r="P48">
+        <f t="shared" si="15"/>
+        <v>0.7953699600184897</v>
+      </c>
+      <c r="Q48">
+        <f t="shared" si="21"/>
+        <v>0.16129032258064516</v>
+      </c>
+      <c r="R48">
+        <f t="shared" si="22"/>
+        <v>0.17142857142857146</v>
+      </c>
+      <c r="S48">
+        <f t="shared" si="23"/>
+        <v>0.47243783712669385</v>
+      </c>
+      <c r="T48">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="U48">
+        <f t="shared" si="25"/>
+        <v>0.64895118999596602</v>
+      </c>
+      <c r="V48">
+        <f t="shared" si="26"/>
+        <v>0.81912144702842382</v>
+      </c>
+      <c r="W48">
+        <f t="shared" si="27"/>
+        <v>0.7458393151486149</v>
+      </c>
+      <c r="X48">
+        <f t="shared" si="28"/>
+        <v>2.0930232558139536E-4</v>
+      </c>
+      <c r="Y48">
+        <f t="shared" si="29"/>
+        <v>8.1221198156682037E-2</v>
+      </c>
+      <c r="Z48">
+        <f t="shared" si="30"/>
+        <v>0.58406654935210378</v>
+      </c>
+      <c r="AA48">
+        <f t="shared" si="31"/>
+        <v>1</v>
+      </c>
+      <c r="AC48">
+        <f t="shared" si="16"/>
+        <v>1.9766936392417995</v>
+      </c>
+      <c r="AD48">
+        <f t="shared" si="17"/>
+        <v>2.2242855835291127</v>
+      </c>
+      <c r="AE48">
+        <f t="shared" si="18"/>
+        <v>1.9766936392417995</v>
+      </c>
+      <c r="AF48">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG48">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="49" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B49">
         <v>200040</v>
       </c>
@@ -2778,8 +6047,76 @@
       <c r="M49">
         <v>176.49</v>
       </c>
+      <c r="P49">
+        <f t="shared" si="15"/>
+        <v>0.27257954605021756</v>
+      </c>
+      <c r="Q49">
+        <f t="shared" si="21"/>
+        <v>9.6774193548387094E-2</v>
+      </c>
+      <c r="R49">
+        <f t="shared" si="22"/>
+        <v>0.49591836734693878</v>
+      </c>
+      <c r="S49">
+        <f t="shared" si="23"/>
+        <v>0.55663728456782002</v>
+      </c>
+      <c r="T49">
+        <f t="shared" si="24"/>
+        <v>0.54545454545454541</v>
+      </c>
+      <c r="U49">
+        <f t="shared" si="25"/>
+        <v>0.88987494957644209</v>
+      </c>
+      <c r="V49">
+        <f t="shared" si="26"/>
+        <v>0.33979328165374678</v>
+      </c>
+      <c r="W49">
+        <f t="shared" si="27"/>
+        <v>0.23539107779018453</v>
+      </c>
+      <c r="X49">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="Y49">
+        <f t="shared" si="29"/>
+        <v>5.0835253456221197E-2</v>
+      </c>
+      <c r="Z49">
+        <f t="shared" si="30"/>
+        <v>0.76483762597984317</v>
+      </c>
+      <c r="AA49">
+        <f t="shared" si="31"/>
+        <v>0.93294954283779219</v>
+      </c>
+      <c r="AC49">
+        <f t="shared" si="16"/>
+        <v>1.8323938262545001</v>
+      </c>
+      <c r="AD49">
+        <f t="shared" si="17"/>
+        <v>2.2350784769155934</v>
+      </c>
+      <c r="AE49">
+        <f t="shared" si="18"/>
+        <v>1.8323938262545001</v>
+      </c>
+      <c r="AF49">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG49">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="50" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B50">
         <v>345026</v>
       </c>
@@ -2816,8 +6153,76 @@
       <c r="M50">
         <v>86.582999999999998</v>
       </c>
+      <c r="P50">
+        <f t="shared" si="15"/>
+        <v>0.96349244926065181</v>
+      </c>
+      <c r="Q50">
+        <f t="shared" si="21"/>
+        <v>0.12903225806451613</v>
+      </c>
+      <c r="R50">
+        <f t="shared" si="22"/>
+        <v>0.31020408163265312</v>
+      </c>
+      <c r="S50">
+        <f t="shared" si="23"/>
+        <v>0.65267727930535457</v>
+      </c>
+      <c r="T50">
+        <f t="shared" si="24"/>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="U50">
+        <f t="shared" si="25"/>
+        <v>0.67728922952803539</v>
+      </c>
+      <c r="V50">
+        <f t="shared" si="26"/>
+        <v>4.7803617571059415E-2</v>
+      </c>
+      <c r="W50">
+        <f t="shared" si="27"/>
+        <v>0.28111873238687729</v>
+      </c>
+      <c r="X50">
+        <f t="shared" si="28"/>
+        <v>3.7375415282392029E-2</v>
+      </c>
+      <c r="Y50">
+        <f t="shared" si="29"/>
+        <v>7.3444700460829501E-2</v>
+      </c>
+      <c r="Z50">
+        <f t="shared" si="30"/>
+        <v>0.18892977123660215</v>
+      </c>
+      <c r="AA50">
+        <f t="shared" si="31"/>
+        <v>0.15228320612675506</v>
+      </c>
+      <c r="AC50">
+        <f t="shared" si="16"/>
+        <v>1.5098020081593098</v>
+      </c>
+      <c r="AD50">
+        <f t="shared" si="17"/>
+        <v>2.5185530991105831</v>
+      </c>
+      <c r="AE50">
+        <f t="shared" si="18"/>
+        <v>1.5098020081593098</v>
+      </c>
+      <c r="AF50">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG50">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="51" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B51">
         <v>159173</v>
       </c>
@@ -2854,8 +6259,76 @@
       <c r="M51">
         <v>139.797</v>
       </c>
+      <c r="P51">
+        <f t="shared" si="15"/>
+        <v>7.7832897301367193E-2</v>
+      </c>
+      <c r="Q51">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="R51">
+        <f t="shared" si="22"/>
+        <v>0.68571428571428561</v>
+      </c>
+      <c r="S51">
+        <f t="shared" si="23"/>
+        <v>0.14748059465859756</v>
+      </c>
+      <c r="T51">
+        <f t="shared" si="24"/>
+        <v>1</v>
+      </c>
+      <c r="U51">
+        <f t="shared" si="25"/>
+        <v>0.34721661960467926</v>
+      </c>
+      <c r="V51">
+        <f t="shared" si="26"/>
+        <v>0.16020671834625322</v>
+      </c>
+      <c r="W51">
+        <f t="shared" si="27"/>
+        <v>0.99787313234433983</v>
+      </c>
+      <c r="X51">
+        <f t="shared" si="28"/>
+        <v>1.0382059800664453E-3</v>
+      </c>
+      <c r="Y51">
+        <f t="shared" si="29"/>
+        <v>0.25403225806451613</v>
+      </c>
+      <c r="Z51">
+        <f t="shared" si="30"/>
+        <v>0.61446168613021912</v>
+      </c>
+      <c r="AA51">
+        <f t="shared" si="31"/>
+        <v>0.61434265023834955</v>
+      </c>
+      <c r="AC51">
+        <f t="shared" si="16"/>
+        <v>1.8599737769002005</v>
+      </c>
+      <c r="AD51">
+        <f t="shared" si="17"/>
+        <v>2.3788872091780746</v>
+      </c>
+      <c r="AE51">
+        <f t="shared" si="18"/>
+        <v>1.8599737769002005</v>
+      </c>
+      <c r="AF51">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG51">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B52">
         <v>346397</v>
       </c>
@@ -2892,8 +6365,76 @@
       <c r="M52">
         <v>88.054000000000002</v>
       </c>
+      <c r="P52">
+        <f t="shared" si="15"/>
+        <v>0.97002578068783452</v>
+      </c>
+      <c r="Q52">
+        <f t="shared" si="21"/>
+        <v>0.16129032258064516</v>
+      </c>
+      <c r="R52">
+        <f t="shared" si="22"/>
+        <v>0.10612244897959182</v>
+      </c>
+      <c r="S52">
+        <f t="shared" si="23"/>
+        <v>0.133008814629654</v>
+      </c>
+      <c r="T52">
+        <f t="shared" si="24"/>
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="U52">
+        <f t="shared" si="25"/>
+        <v>0.30264219443323914</v>
+      </c>
+      <c r="V52">
+        <f t="shared" si="26"/>
+        <v>0.18992248062015507</v>
+      </c>
+      <c r="W52">
+        <f t="shared" si="27"/>
+        <v>0.9606529483702877</v>
+      </c>
+      <c r="X52">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="Y52">
+        <f t="shared" si="29"/>
+        <v>0.16474654377880185</v>
+      </c>
+      <c r="Z52">
+        <f t="shared" si="30"/>
+        <v>0.16333386658134699</v>
+      </c>
+      <c r="AA52">
+        <f t="shared" si="31"/>
+        <v>0.16505596221139737</v>
+      </c>
+      <c r="AC52">
+        <f t="shared" si="16"/>
+        <v>1.5913693348872802</v>
+      </c>
+      <c r="AD52">
+        <f t="shared" si="17"/>
+        <v>2.574126329756643</v>
+      </c>
+      <c r="AE52">
+        <f t="shared" si="18"/>
+        <v>1.5913693348872802</v>
+      </c>
+      <c r="AF52">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG52">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="53" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B53">
         <v>247133</v>
       </c>
@@ -2930,8 +6471,76 @@
       <c r="M53">
         <v>148.654</v>
       </c>
+      <c r="P53">
+        <f t="shared" si="15"/>
+        <v>0.49699543000376467</v>
+      </c>
+      <c r="Q53">
+        <f t="shared" si="21"/>
+        <v>6.4516129032258063E-2</v>
+      </c>
+      <c r="R53">
+        <f t="shared" si="22"/>
+        <v>0.34693877551020419</v>
+      </c>
+      <c r="S53">
+        <f t="shared" si="23"/>
+        <v>0.344823049598737</v>
+      </c>
+      <c r="T53">
+        <f t="shared" si="24"/>
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="U53">
+        <f t="shared" si="25"/>
+        <v>0.62938684953610324</v>
+      </c>
+      <c r="V53">
+        <f t="shared" si="26"/>
+        <v>0.12015503875968991</v>
+      </c>
+      <c r="W53">
+        <f t="shared" si="27"/>
+        <v>0.72244377093635359</v>
+      </c>
+      <c r="X53">
+        <f t="shared" si="28"/>
+        <v>9.4352159468438553E-3</v>
+      </c>
+      <c r="Y53">
+        <f t="shared" si="29"/>
+        <v>4.9395161290322578E-2</v>
+      </c>
+      <c r="Z53">
+        <f t="shared" si="30"/>
+        <v>0.29771236602143658</v>
+      </c>
+      <c r="AA53">
+        <f t="shared" si="31"/>
+        <v>0.69124836107565535</v>
+      </c>
+      <c r="AC53">
+        <f t="shared" si="16"/>
+        <v>1.5481830680597051</v>
+      </c>
+      <c r="AD53">
+        <f t="shared" si="17"/>
+        <v>2.3617881454687568</v>
+      </c>
+      <c r="AE53">
+        <f t="shared" si="18"/>
+        <v>1.5481830680597051</v>
+      </c>
+      <c r="AF53">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG53">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="54" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B54">
         <v>206636</v>
       </c>
@@ -2968,8 +6577,76 @@
       <c r="M54">
         <v>107.98099999999999</v>
       </c>
+      <c r="P54">
+        <f t="shared" si="15"/>
+        <v>0.30401197062621815</v>
+      </c>
+      <c r="Q54">
+        <f t="shared" si="21"/>
+        <v>6.4516129032258063E-2</v>
+      </c>
+      <c r="R54">
+        <f t="shared" si="22"/>
+        <v>0.91428571428571448</v>
+      </c>
+      <c r="S54">
+        <f t="shared" si="23"/>
+        <v>0.60136824102091835</v>
+      </c>
+      <c r="T54">
+        <f t="shared" si="24"/>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="U54">
+        <f t="shared" si="25"/>
+        <v>0.64068172650262201</v>
+      </c>
+      <c r="V54">
+        <f t="shared" si="26"/>
+        <v>0.18863049095607234</v>
+      </c>
+      <c r="W54">
+        <f t="shared" si="27"/>
+        <v>0</v>
+      </c>
+      <c r="X54">
+        <f t="shared" si="28"/>
+        <v>1</v>
+      </c>
+      <c r="Y54">
+        <f t="shared" si="29"/>
+        <v>8.8421658986175114E-2</v>
+      </c>
+      <c r="Z54">
+        <f t="shared" si="30"/>
+        <v>0.49448088305871057</v>
+      </c>
+      <c r="AA54">
+        <f t="shared" si="31"/>
+        <v>0.33808295779172853</v>
+      </c>
+      <c r="AC54">
+        <f t="shared" si="16"/>
+        <v>1.8202866984964519</v>
+      </c>
+      <c r="AD54">
+        <f t="shared" si="17"/>
+        <v>2.2661405982664373</v>
+      </c>
+      <c r="AE54">
+        <f t="shared" si="18"/>
+        <v>1.8202866984964519</v>
+      </c>
+      <c r="AF54">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG54">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="55" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B55">
         <v>276146</v>
       </c>
@@ -3005,6 +6682,97 @@
       </c>
       <c r="M55">
         <v>139.31</v>
+      </c>
+      <c r="P55">
+        <f t="shared" si="15"/>
+        <v>0.63525330359738286</v>
+      </c>
+      <c r="Q55">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="R55">
+        <f t="shared" si="22"/>
+        <v>0.46326530612244904</v>
+      </c>
+      <c r="S55">
+        <f t="shared" si="23"/>
+        <v>0.22247072753585054</v>
+      </c>
+      <c r="T55">
+        <f t="shared" si="24"/>
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="U55">
+        <f t="shared" si="25"/>
+        <v>0.37736990722065339</v>
+      </c>
+      <c r="V55">
+        <f t="shared" si="26"/>
+        <v>0.24806201550387597</v>
+      </c>
+      <c r="W55">
+        <f t="shared" si="27"/>
+        <v>0.92449619822406559</v>
+      </c>
+      <c r="X55">
+        <f t="shared" si="28"/>
+        <v>4.7009966777408643E-4</v>
+      </c>
+      <c r="Y55">
+        <f t="shared" si="29"/>
+        <v>8.4101382488479245E-2</v>
+      </c>
+      <c r="Z55">
+        <f t="shared" si="30"/>
+        <v>0.12973924172132459</v>
+      </c>
+      <c r="AA55">
+        <f t="shared" si="31"/>
+        <v>0.61011400835308738</v>
+      </c>
+      <c r="AC55">
+        <f t="shared" si="16"/>
+        <v>1.7172308166620376</v>
+      </c>
+      <c r="AD55">
+        <f t="shared" si="17"/>
+        <v>2.3958329404701959</v>
+      </c>
+      <c r="AE55">
+        <f t="shared" si="18"/>
+        <v>1.7172308166620376</v>
+      </c>
+      <c r="AF55">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AG55">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AE56">
+        <f>SUM(AE5:AE55)</f>
+        <v>86.929696532993802</v>
+      </c>
+      <c r="AF56">
+        <f>SUM(AF5:AF55)</f>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="58" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="P58" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="Q59" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>